<commit_message>
update final version data
</commit_message>
<xml_diff>
--- a/02-data/02-gt-artifacts.xlsx
+++ b/02-data/02-gt-artifacts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuxiaoran/Downloads/icsa-2025-replication-package/02-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6931E5B-BE0D-8B4F-9327-83896AA10443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E93309-EA34-0242-B9AA-62C812353C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="axial-coding" sheetId="1" r:id="rId1"/>
@@ -165,7 +165,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>: Env</t>
@@ -190,7 +189,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>: baseEnv</t>
@@ -267,7 +265,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> for RL environment, NO FILES</t>
@@ -364,7 +361,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -744,7 +740,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, </t>
@@ -764,7 +759,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, 
@@ -785,7 +779,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -937,7 +930,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, </t>
@@ -957,7 +949,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>, 
@@ -1120,7 +1111,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Basically:
@@ -1944,7 +1934,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>tianshou/highlevel/config.py
@@ -2286,7 +2275,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">: 
@@ -2910,7 +2898,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -2932,7 +2919,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> class Logger
@@ -3503,7 +3489,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3542,7 +3527,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3567,7 +3551,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3596,7 +3579,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (example)
@@ -3620,7 +3602,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3660,7 +3641,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3686,7 +3666,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">You </t>
@@ -3705,7 +3684,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>. An Algorithm typically holds a neural network for computing actions, called policy, the RL environment that you want to optimize against, a loss function, an optimizer, and some code describing the algorithm’s execution logic, like determining when to collect samples, when to update your model, etc..</t>
@@ -3727,7 +3705,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3754,7 +3731,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -3776,7 +3752,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3812,7 +3787,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3840,7 +3814,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3864,7 +3837,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3892,7 +3864,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3917,7 +3888,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">create env, agent, checkpoint, logging
@@ -3949,7 +3919,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -3976,7 +3945,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4017,7 +3985,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>rl_zoo3/hyperparams_opt.py
@@ -4048,7 +4015,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4084,7 +4050,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4120,7 +4085,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4144,7 +4108,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4173,7 +4136,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4202,7 +4164,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (example)
@@ -4230,7 +4191,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4253,7 +4213,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4279,7 +4238,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">You </t>
@@ -4298,7 +4256,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. An Algorithm typically holds a neural network for computing actions, called policy, the RL environment that you want to optimize against, a loss function, an optimizer, and some code describing the algorithm’s execution logic, like determining when to collect samples, when to update your model, etc..
@@ -4321,7 +4278,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -4349,7 +4305,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4385,7 +4340,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4423,7 +4377,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4447,7 +4400,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4474,7 +4426,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4516,7 +4467,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4544,7 +4494,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4580,7 +4529,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4602,7 +4550,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4636,7 +4583,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -4659,7 +4605,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4696,7 +4641,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4740,7 +4684,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -4762,7 +4705,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4794,7 +4736,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4831,7 +4772,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">def _run_train_phase(self, statistics):
@@ -4856,7 +4796,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4884,7 +4823,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4908,7 +4846,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> with the configuration given at construction.
@@ -4932,7 +4869,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4954,7 +4890,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -4982,7 +4917,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5010,7 +4944,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -5036,7 +4969,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5057,7 +4989,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5082,7 +5013,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5104,7 +5034,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5141,7 +5070,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5172,7 +5100,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> Config, lightweight configuration framework
@@ -5195,7 +5122,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5221,7 +5147,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5252,7 +5177,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5275,7 +5199,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5298,7 +5221,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5321,7 +5243,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5345,7 +5266,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5379,7 +5299,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5401,7 +5320,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5426,7 +5344,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5474,7 +5391,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5504,7 +5420,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5526,7 +5441,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>):
@@ -5573,7 +5487,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5606,7 +5519,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">)  
@@ -5627,7 +5539,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5659,7 +5570,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5682,7 +5592,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5724,7 +5633,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The first of these is Anakin, which can be used when environments are written in JAX. This enables end-to-end JIT compilation of the full MARL training loop for fast experiment run times on hardware accelerators. The second is Sebulba, which can be used when environments are not written in JAX. Sebulba is particularly useful when running RL experiments where a hardware accelerator can interact with many CPU cores at a time.</t>
@@ -5746,7 +5654,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5768,7 +5675,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5796,7 +5702,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5826,7 +5731,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5853,7 +5757,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5874,7 +5777,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -5896,7 +5798,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5925,7 +5826,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -5951,7 +5851,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -5982,7 +5881,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6016,7 +5914,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6040,7 +5937,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6062,7 +5958,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6088,7 +5983,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6113,7 +6007,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6144,7 +6037,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -6167,7 +6059,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6190,7 +6081,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6211,7 +6101,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6238,7 +6127,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6263,7 +6151,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6284,7 +6171,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6312,7 +6198,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -6338,7 +6223,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6359,7 +6243,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6384,7 +6267,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6406,7 +6288,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6438,7 +6319,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6465,7 +6345,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6489,7 +6368,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6514,7 +6392,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6543,7 +6420,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -6566,7 +6442,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6591,7 +6466,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6620,7 +6494,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6641,7 +6514,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6666,7 +6538,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6696,7 +6567,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6737,7 +6607,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6762,7 +6631,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6784,7 +6652,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6810,7 +6677,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6839,7 +6705,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6869,7 +6734,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6896,7 +6760,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6917,7 +6780,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6942,7 +6804,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -6970,7 +6831,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -7044,7 +6904,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7086,7 +6945,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -7119,7 +6977,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7143,7 +7000,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7172,7 +7028,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7195,7 +7050,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7223,7 +7077,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -7252,7 +7105,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>ml-agents-envs/mlagents_envs/environment.py</t>
@@ -7274,7 +7126,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7298,7 +7149,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7322,7 +7172,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7343,7 +7192,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7377,7 +7225,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7405,7 +7252,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7428,7 +7274,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7453,7 +7298,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7476,7 +7320,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7511,7 +7354,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7543,7 +7385,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -7580,7 +7421,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -7602,7 +7442,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7628,7 +7467,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7650,7 +7488,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7671,7 +7508,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">: The action manager that processes the raw actions sent to the environment and converts them to low-level commands that are sent to the simulation. It can be configured to accept raw actions at different levels of abstraction. For example, in case of a robotic arm, the raw actions can be joint torques, joint positions, or end-effector poses. Similarly for a mobile base, it can be  the joint torques, or the desired velocity of the floating base.
@@ -7692,7 +7528,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7713,7 +7548,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -7735,7 +7569,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7755,7 +7588,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -7778,7 +7610,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -7808,7 +7639,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Environment
@@ -7833,7 +7663,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7860,7 +7689,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7891,7 +7719,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7913,7 +7740,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7943,7 +7769,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7971,7 +7796,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -7994,7 +7818,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8028,7 +7851,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8051,7 +7873,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8075,7 +7896,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8099,7 +7919,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8124,7 +7943,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8152,7 +7970,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8182,7 +7999,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8208,7 +8024,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8238,7 +8053,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8265,7 +8079,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8291,7 +8104,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8326,7 +8138,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8358,7 +8169,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8391,7 +8201,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8421,7 +8230,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8444,7 +8252,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8469,7 +8276,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8493,7 +8299,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8527,7 +8332,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -8561,7 +8365,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8589,7 +8392,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8618,7 +8420,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8649,7 +8450,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8687,7 +8487,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8737,7 +8536,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8776,7 +8574,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8797,7 +8594,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8831,7 +8627,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">examples/checkpointing/reload_experiment.py
@@ -8855,7 +8650,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8887,7 +8681,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8914,7 +8707,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8945,7 +8737,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -8972,7 +8763,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9000,7 +8790,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9021,7 +8810,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> to your isaacgymenvs tasks:
@@ -9046,7 +8834,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9070,7 +8857,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9094,7 +8880,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9133,7 +8918,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9159,7 +8943,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9191,7 +8974,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9218,7 +9000,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9244,7 +9025,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9268,7 +9048,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9276,7 +9055,30 @@
 Run rendering without stepping through the physics.
 By convention, if mode is:
 human: Render to the current display and return nothing. Usually for human consumption.
-rgb_array: Return a numpy.ndarray with shape (x, y, 3), representing RGB values for an x-by-y pixel image, suitable for turning into a video.</t>
+rgb_array: Return a numpy.ndarray with shape (x, y, 3), representing RGB values for an x-by-y pixel image, suitable for turning into a video.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacLab/blob/main/source/isaaclab_contrib/isaaclab_contrib/sensors/tacsl_sensor/visuotactile_render.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+class GelsightRender:
+    """Class to handle GelSight rendering using the Taxim example-based approach from :cite:t:`si2022taxim`.
+</t>
     </r>
   </si>
   <si>
@@ -9299,7 +9101,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">         
@@ -9324,7 +9125,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9352,7 +9152,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9375,7 +9174,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9398,7 +9196,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -9420,7 +9217,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9456,7 +9252,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -9480,7 +9275,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9505,7 +9299,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9537,7 +9330,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9564,7 +9356,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9588,7 +9379,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9610,7 +9400,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9634,7 +9423,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9656,7 +9444,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9678,7 +9465,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9701,7 +9487,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9727,7 +9512,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9749,7 +9533,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9772,7 +9555,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9796,7 +9578,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9823,7 +9604,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9860,7 +9640,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9883,7 +9662,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9910,7 +9688,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9936,7 +9713,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9964,7 +9740,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -9987,7 +9762,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -10018,7 +9792,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10044,7 +9817,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10071,7 +9843,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10102,7 +9873,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10143,7 +9913,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10174,7 +9943,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10198,7 +9966,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10223,7 +9990,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10248,7 +10014,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10270,7 +10035,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10292,7 +10056,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10318,7 +10081,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  
@@ -10354,7 +10116,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Logging &amp; Saving
@@ -10374,7 +10135,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. You can change the saved log location here:
@@ -10395,7 +10155,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -10417,7 +10176,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10445,7 +10203,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10473,7 +10230,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">(BaseLogger):
@@ -10508,7 +10264,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(BaseLogger):
@@ -10538,7 +10293,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10564,7 +10318,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10593,7 +10346,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10619,7 +10371,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10644,7 +10395,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10682,7 +10432,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10705,7 +10454,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10730,7 +10478,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">..)
@@ -10754,7 +10501,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10778,7 +10524,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10801,7 +10546,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10828,7 +10572,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10852,7 +10595,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10897,7 +10639,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10918,7 +10659,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -10939,7 +10679,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> (
@@ -10972,7 +10711,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -10995,7 +10733,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -11015,7 +10752,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(
@@ -11070,7 +10806,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
@@ -11093,7 +10828,6 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> and log statistics.
@@ -34117,10 +33851,10 @@
       <c r="C22" s="19" t="s">
         <v>536</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="18" t="s">
         <v>537</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="18" t="s">
         <v>538</v>
       </c>
       <c r="F22" s="19" t="s">
@@ -34135,7 +33869,7 @@
       <c r="I22" s="19" t="s">
         <v>542</v>
       </c>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="18" t="s">
         <v>543</v>
       </c>
       <c r="K22" s="19" t="s">

</xml_diff>

<commit_message>
update the data and rerun the charts & stats
</commit_message>
<xml_diff>
--- a/02-data/02-gt-artifacts.xlsx
+++ b/02-data/02-gt-artifacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuxiaoran/Downloads/icsa-2025-replication-package/02-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E93309-EA34-0242-B9AA-62C812353C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A8DA2A-FF84-8440-8B8F-04945F3F4F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="631">
   <si>
     <t>Components</t>
   </si>
@@ -3474,6 +3474,42 @@
     <t>use experiment logger results, generate metrics report, and plot</t>
   </si>
   <si>
+    <t>Development Team</t>
+  </si>
+  <si>
+    <t>Farama Foundation</t>
+  </si>
+  <si>
+    <t>Unity</t>
+  </si>
+  <si>
+    <t>NVIDIA</t>
+  </si>
+  <si>
+    <t>Google DeepMind</t>
+  </si>
+  <si>
+    <t>Research Team at InstaDeep.</t>
+  </si>
+  <si>
+    <t>Antonin Raffin - German Aerospace Center (DLR)</t>
+  </si>
+  <si>
+    <t>RISELab at UCB, now company Anyscale.</t>
+  </si>
+  <si>
+    <t>small research team</t>
+  </si>
+  <si>
+    <t>Company: Meta</t>
+  </si>
+  <si>
+    <t>Company: Google</t>
+  </si>
+  <si>
+    <t>Research: Tsinghua University</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <u/>
@@ -8315,6 +8351,398 @@
   </si>
   <si>
     <t>Data Persistence</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Unity-Technologies/ml-agents/blob/develop/ml-agents/mlagents/trainers/policy/checkpoint_manager.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Unity-Technologies/ml-agents/blob/develop/ml-agents/mlagents/trainers/model_saver/model_saver.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Unity-Technologies/ml-agents/blob/develop/com.unity.ml-agents/Runtime/EnvironmentParameters.cs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacGymEnvs/blob/main/docs/domain_randomization.md?plain=1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+We provide two interfaces to add 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>domain randomization</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to your isaacgymenvs tasks:
+Adding domain randomization parameters to your task's YAML config
+Directly calling the apply_randomizations class method
+Provided your task inherits from our VecTask class, you have great flexibility in choosing when to randomize and what distributions to sample, and can even change the entire domain randomization dictionary at every call to apply_randomizations if you wish.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://isaac-sim.github.io/IsaacLab/main/source/tutorials/03_envs/create_direct_rl_env.html</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+In Isaac Lab, the domain randomization configuration 
+uses the configclass module to specify a configuration class 
+consisting of EventTermCfg variables.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacLab/blob/main/source/isaaclab/isaaclab/managers/curriculum_manager.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+CurriculumManager:The curriculum manager updates various quantities of the environment subject to a training curriculum by calling a list of terms. 
+These help stabilize learning by progressively making the learning tasks harder as the agent improves.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Farama-Foundation/Arcade-Learning-Environment/blob/master/src/ale/ale_interface.hpp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+src/ale/ale_interface.hpp
+DifficultyVect getAvailableDifficulties() const;
+void setDifficulty(difficulty_t m);
+difficulty_t getDifficulty() 
+ModeVect getAvailableModes() const;
+void setMode(game_mode_t m);
+game_mode_t getMode()</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/instadeepai/jumanji/blob/main/jumanji/training/loggers.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+class Logger(AbstractContextManager)
+write, close, upload_checkpoint(self) -&gt; None:
+        """Uploads a checkpoint when exiting the logger.
+_save_and_upload_checkpoint(self) -&gt; None:
+        """Grabs the `training_state` variable from within the context manager, pickles it and
+        saves it. This will break if the desired variable to checkpoint is not called
+        `training_state`.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/DLR-RM/stable-baselines3/blob/master/stable_baselines3/common/callbacks.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+stable_baselines3/common/callbacks.py
+class CheckpointCallback(BaseCallback):
+    """
+    Callback for saving a model every ``save_freq`` calls
+    to ``env.step()``.
+    By default, it only saves model checkpoints,
+    you need to pass ``save_replay_buffer=True``,
+    and ``save_vecnormalize=True`` to also save replay buffer checkpoints
+    and normalization statistics checkpoints.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/DLR-RM/rl-baselines3-zoo/blob/master/rl_zoo3/utils.py 	"def get_model_path(
+    exp_id: int,
+    folder: str,
+    algo: str,
+    env_name: EnvironmentName,
+    load_best: bool = False,
+    load_checkpoint: str | None = None,
+    load_last_checkpoint: bool = False,
+) -&gt; tuple[str, str, str]:
+    if exp_id == 0:
+        exp_id = get_latest_run_id(os.path.join(folder, algo), env_name)
+        print(f""Loading latest experiment, id={exp_id}"")"</t>
+  </si>
+  <si>
+    <t>https://github.com/ray-project/ray/blob/master/rllib/utils/checkpoints.py 
+rllib/utils/checkpoints.py
+class Checkpointable(abc.ABC):
+    """Abstract base class for a component of RLlib that can be checkpointed to disk</t>
+  </si>
+  <si>
+    <t>https://github.com/google-deepmind/acme/blob/master/acme/tf/savers.py 	"class Checkpointer:
+  """"""Convenience class for periodically checkpointing.
+ def save(self, force: bool = False) -&gt; bool:
+    """"""Save the checkpoint if it's the appropriate time, otherwise no-ops.
+ def restore(self):
+    """"""Restore from most recent checkpoint.""""""
+class CheckpointingRunner(core.Worker):
+  """"""Wrap an object and expose a run method which checkpoints periodically.
+"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">UseRLlib (Ray), </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/ray-project/ray/blob/master/python/ray/tune/trainable/trainable_fn_utils.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/facebookresearch/BenchMARL/tree/main/examples/checkpointing	
+checkpointing folder, including reload and resume files</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/tree/develop/mava/utils</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">checkpointing.py
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utils have (i) checkpointing (ii) logger for logging and reporting (external)
+checkpointing: 
+class Checkpointer:
+    """Model checkpointer for saving and restoring the `learner_state`."""
+    def __init__(
+        self,
+        model_name: str,
+        metadata: Optional[Dict] = None,
+        rel_dir: str = "checkpoints",
+        checkpoint_uid: Optional[str] = None,
+        save_interval_steps: int = 1,
+        max_to_keep: Optional[int] = 1,
+        keep_period: Optional[int] = None,
+    ):
+        """Initialise the checkpointer tool</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/checkpointer.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+dopamine/discrete_domains/checkpointer.py
+"""A checkpointing mechanism for Dopamine agents.
+from absl import logging
+from dopamine.discrete_domains import atari_lib
+from dopamine.discrete_domains import checkpointer
+from dopamine.discrete_domains import iteration_statistics
+from dopamine.discrete_domains import logger
+class Checkpointer(object):
+  """Class for managing checkpoints for Dopamine agents."""</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">class Persistence(ABC):
+    @abstractmethod
+    def persist(self, event: PersistEvent, world: World) -&gt; None:
+        pass
+    @abstractmethod
+    def restore(self, event: RestoreEvent, world: World) -&gt; None:
+        pass
+class PersistenceGroup(Persistence):
+https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/persistence.py  </t>
   </si>
   <si>
     <r>
@@ -8896,6 +9324,362 @@
     <t>Monitoring &amp; Visualization</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Farama-Foundation/Gymnasium/tree/main/gymnasium/utils</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+utils module have: record &amp; save video
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Farama-Foundation/Gymnasium/blob/main/gymnasium/logger.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+Logger
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Farama-Foundation/Gymnasium/blob/main/gymnasium/wrappers/utils.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+wrapper utils</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/Farama-Foundation/PettingZoo/tree/master/pettingzoo/utils 	utils folder: logger, save, total reward...</t>
+  </si>
+  <si>
+    <t>"https://github.com/Unity-Technologies/ml-agents/blob/develop/ml-agents-envs/mlagents_envs/logging_util.py 
+https://github.com/Unity-Technologies/ml-agents/blob/develop/ml-agents/mlagents/trainers/stats.py "
+   """
+    Create a logger with the specified name. The logger will use the log level
+    specified by set_log_level()
+    """, 
+class StatsSummary(NamedTuple):
+class StatsWriter(abc.ABC):
+    """
+    A StatsWriter abstract class. A StatsWriter takes in a category, key, scalar value, and step
+    and writes it out by some method.
+    """</t>
+  </si>
+  <si>
+    <t>code are mainly in the vec_task, but not a standalone module. also, only use the logger/reporter by calling python libs</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacLab/blob/main/source/isaaclab/isaaclab/envs/manager_based_rl_env.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacLab/blob/main/source/isaaclab_contrib/isaaclab_contrib/sensors/tacsl_sensor/visuotactile_render.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+class GelsightRender:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/isaac-sim/IsaacLab/blob/main/source/isaaclab/isaaclab/managers/recorder_manager.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/google-deepmind/dm_control/tree/main/dm_control/viewer	The dm_control.viewer library can be used to visualize and interact with a control environment. The following example shows how to launch the viewer with an environment from the Control Suite:	renderer, viewer, logger</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/google-deepmind/lab/tree/master/engine/code/renderercommon</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/google-deepmind/lab/blob/master/game_scripts/common/log.lua</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.
+multiple rendereer; logger files; and recording files</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/instadeepai/jumanji/blob/main/jumanji/env.py ;
+https://github.com/instadeepai/jumanji/blob/main/jumanji/viewer.py 
+https://github.com/instadeepai/jumanji/blob/main/jumanji/training/loggers.py </t>
+  </si>
+  <si>
+    <t>https://github.com/DLR-RM/stable-baselines3/tree/master/stable_baselines3/common	
+logger.py monitor.py save_util.py</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/DLR-RM/rl-baselines3-zoo/blob/master/rl_zoo3/record_training.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/DLR-RM/rl-baselines3-zoo/blob/master/rl_zoo3/record_video.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/DLR-RM/rl-baselines3-zoo/tree/master/rl_zoo3/plots</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/ray-project/ray/tree/master/rllib/utils
+have metrics for reporting, error for logging.</t>
+  </si>
+  <si>
+    <t>"https://github.com/google-deepmind/acme/tree/master/acme/utils/loggers
+https://github.com/google-deepmind/acme/blob/master/acme/wrappers/video.py
+utils/loggers
+wrappers/video.py</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Use RLLib (Ray): </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/ray-project/ray/blob/master/python/ray/tune/progress_reporter.py</t>
+    </r>
+  </si>
+  <si>
+    <t>"class Logger:
+    def __init__(
+        self,
+        experiment_name: str,
+        folder_name: str,
+        experiment_config,
+        algorithm_name: str,
+        environment_name: str,
+        task_name: str,
+        model_name: str,
+        group_map: Dict[str, List[str]],
+        seed: int,
+        project_name: str,
+        wandb_extra_kwargs: Dict[str, Any],
+    ):"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/utils/logger.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+class MavaLogger:
+    def __init__(
+        self,
+        config: DictConfig,
+        custom_metrics_fn: Callable[[Metrics], Metrics] = winrate_custom_metric,
+    ) -&gt; None:
+        """The main logger for Mava systems.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">https://github.com/google/dopamine/tree/master/dopamine/utils 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Utils has bar_plotter, line_plotter, agent_visualizer, etc.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/logger.py 
+tianshou/highlevel/logger.py
+from tianshou.utils import BaseLogger, TensorboardLogger, WandbLogger
+"""A logger that relies on tensorboard SummaryWriter by default to visualize and log statistics.</t>
+  </si>
+  <si>
     <t>Renderer</t>
   </si>
   <si>
@@ -9167,7 +9951,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>https://github.com/Farama-Foundation/Arcade-Learning-Environment/blob/master/src/ale/python/env.py</t>
+      <t>https://github.com/Farama-Foundation/Arcade-Learning-Environment/blob/master/src/ale/common/ScreenSDL.hpp</t>
     </r>
     <r>
       <rPr>
@@ -9177,7 +9961,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> 
-render()</t>
+A method called render() that displays frames</t>
     </r>
   </si>
   <si>
@@ -9745,34 +10529,6 @@
       <t xml:space="preserve"> 
 isaacgymenvs/tasks/amp/poselib/poselib/core/backend/logger.py  
 import logging
-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>https://github.com/isaac-sim/IsaacGymEnvs/blob/main/isaacgymenvs/learning/common_agent.py</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-from tensorboardX import SummaryWriter
-self.eval_summary_dir = "./eval_summaries"
-# remove the old directory if it exists
-if os.path.exists(self.eval_summary_dir):
-import shutil
-shutil.rmtree(self.eval_summary_dir)
-self.eval_summaries = SummaryWriter(self.eval_summary_dir, flush_secs=3)
-The SummaryWriter class is your main entry to log data for consumption and visualization by TensorBoard. 
 </t>
     </r>
   </si>
@@ -10207,13 +10963,6 @@
       </rPr>
       <t xml:space="preserve"> 
 mava/utils/logger.py
-class MavaLogger:
-    def __init__(
-        self,
-        config: DictConfig,
-        custom_metrics_fn: Callable[[Metrics], Metrics] = winrate_custom_metric,
-    ) -&gt; None:
-        """The main logger for Mava systems.
 class </t>
     </r>
     <r>
@@ -10834,12 +11583,33 @@
 </t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://www.tensorflow.org/resources/libraries-extensions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -10928,6 +11698,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF474747"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
@@ -10956,6 +11732,27 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
@@ -11152,7 +11949,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -11194,33 +11991,53 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32608,7 +33425,7 @@
       <c r="AA8" s="16"/>
     </row>
     <row r="9" spans="1:27" ht="56" x14ac:dyDescent="0.15">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="33" t="s">
         <v>336</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -32626,7 +33443,7 @@
       </c>
     </row>
     <row r="10" spans="1:27" ht="28" x14ac:dyDescent="0.15">
-      <c r="A10" s="26"/>
+      <c r="A10" s="34"/>
       <c r="B10" s="4" t="s">
         <v>340</v>
       </c>
@@ -32642,7 +33459,7 @@
       </c>
     </row>
     <row r="11" spans="1:27" ht="70" x14ac:dyDescent="0.15">
-      <c r="A11" s="26"/>
+      <c r="A11" s="34"/>
       <c r="B11" s="4" t="s">
         <v>262</v>
       </c>
@@ -32658,7 +33475,7 @@
       </c>
     </row>
     <row r="12" spans="1:27" ht="56" x14ac:dyDescent="0.15">
-      <c r="A12" s="27"/>
+      <c r="A12" s="35"/>
       <c r="B12" s="4" t="s">
         <v>345</v>
       </c>
@@ -32670,13 +33487,13 @@
       <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:27" ht="42" x14ac:dyDescent="0.15">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="33" t="s">
         <v>347</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="33" t="s">
         <v>347</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="33" t="s">
         <v>348</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -32690,9 +33507,9 @@
       </c>
     </row>
     <row r="14" spans="1:27" ht="28" x14ac:dyDescent="0.15">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
       <c r="D14" s="4" t="s">
         <v>351</v>
       </c>
@@ -32704,9 +33521,9 @@
       </c>
     </row>
     <row r="15" spans="1:27" ht="28" x14ac:dyDescent="0.15">
-      <c r="A15" s="26"/>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
+      <c r="A15" s="34"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
       <c r="D15" s="4" t="s">
         <v>354</v>
       </c>
@@ -32718,9 +33535,9 @@
       </c>
     </row>
     <row r="16" spans="1:27" ht="42" x14ac:dyDescent="0.15">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
       <c r="D16" s="8" t="s">
         <v>142</v>
       </c>
@@ -32751,9 +33568,9 @@
       <c r="AA16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="56" x14ac:dyDescent="0.15">
-      <c r="A17" s="26"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
+      <c r="A17" s="34"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
       <c r="D17" s="8" t="s">
         <v>117</v>
       </c>
@@ -32765,11 +33582,11 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="42" x14ac:dyDescent="0.15">
-      <c r="A18" s="26"/>
-      <c r="B18" s="25" t="s">
+      <c r="A18" s="34"/>
+      <c r="B18" s="33" t="s">
         <v>129</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="33" t="s">
         <v>360</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -32783,9 +33600,9 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="28" x14ac:dyDescent="0.15">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
       <c r="D19" s="4" t="s">
         <v>364</v>
       </c>
@@ -32797,7 +33614,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="28" x14ac:dyDescent="0.15">
-      <c r="A20" s="27"/>
+      <c r="A20" s="35"/>
       <c r="B20" s="4" t="s">
         <v>367</v>
       </c>
@@ -32924,7 +33741,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:U34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
@@ -32932,1318 +33749,1516 @@
     <col min="3" max="3" width="31.5" customWidth="1"/>
     <col min="4" max="4" width="35.83203125" customWidth="1"/>
     <col min="5" max="5" width="56.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="42.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="34.83203125" customWidth="1"/>
     <col min="10" max="10" width="32.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="31.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="36" customWidth="1"/>
+    <col min="12" max="13" width="40" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="67.5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="45.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="48.5" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="51" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="71" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="30.6640625" customWidth="1"/>
+    <col min="19" max="19" width="45.5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="41.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="14" x14ac:dyDescent="0.15">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:21" ht="14" x14ac:dyDescent="0.15">
+      <c r="A1" s="17"/>
+      <c r="B1" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="J1" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="L1" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="M1" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="N1" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="O1" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="P1" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="Q1" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="R1" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="S1" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="T1" s="36" t="s">
+        <v>398</v>
+      </c>
+      <c r="U1" s="37"/>
+    </row>
+    <row r="2" spans="1:21" ht="14" x14ac:dyDescent="0.15">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="14" x14ac:dyDescent="0.15">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:21" ht="28" x14ac:dyDescent="0.15">
+      <c r="A3" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="384" x14ac:dyDescent="0.15">
-      <c r="A3" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="18" t="s">
-        <v>387</v>
-      </c>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-    </row>
-    <row r="4" spans="1:20" ht="306" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:21" ht="384" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18" t="s">
-        <v>388</v>
-      </c>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18" t="s">
-        <v>389</v>
-      </c>
-      <c r="M4" s="19" t="s">
-        <v>390</v>
-      </c>
-      <c r="N4" s="18" t="s">
-        <v>391</v>
-      </c>
-      <c r="O4" s="18" t="s">
-        <v>392</v>
-      </c>
-      <c r="P4" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="Q4" s="18" t="s">
-        <v>394</v>
-      </c>
-      <c r="R4" s="18" t="s">
-        <v>395</v>
-      </c>
-      <c r="S4" s="18" t="s">
-        <v>396</v>
-      </c>
-      <c r="T4" s="19" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="280" x14ac:dyDescent="0.15">
+      <c r="B4" s="4"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="21" t="s">
+        <v>399</v>
+      </c>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+    </row>
+    <row r="5" spans="1:21" ht="397" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
         <v>320</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="20" t="s">
-        <v>398</v>
-      </c>
-      <c r="N5" s="20" t="s">
-        <v>399</v>
-      </c>
-      <c r="O5" s="17"/>
-      <c r="P5" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21" t="s">
         <v>400</v>
       </c>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-    </row>
-    <row r="6" spans="1:20" ht="56" x14ac:dyDescent="0.15">
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21" t="s">
+        <v>401</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>402</v>
+      </c>
+      <c r="N5" s="21" t="s">
+        <v>403</v>
+      </c>
+      <c r="O5" s="21" t="s">
+        <v>404</v>
+      </c>
+      <c r="P5" s="21" t="s">
+        <v>405</v>
+      </c>
+      <c r="Q5" s="21" t="s">
+        <v>406</v>
+      </c>
+      <c r="R5" s="21" t="s">
+        <v>407</v>
+      </c>
+      <c r="S5" s="21" t="s">
+        <v>408</v>
+      </c>
+      <c r="T5" s="22" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="345" x14ac:dyDescent="0.15">
       <c r="A6" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="23" t="s">
+        <v>410</v>
+      </c>
+      <c r="N6" s="23" t="s">
+        <v>411</v>
+      </c>
+      <c r="O6" s="20"/>
+      <c r="P6" s="23" t="s">
+        <v>412</v>
+      </c>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
+    </row>
+    <row r="7" spans="1:21" ht="70" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>226</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="19" t="s">
-        <v>401</v>
-      </c>
-      <c r="R6" s="17"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="17"/>
-    </row>
-    <row r="7" spans="1:20" ht="306" x14ac:dyDescent="0.15">
-      <c r="A7" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="18" t="s">
-        <v>402</v>
-      </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="18" t="s">
-        <v>403</v>
-      </c>
-      <c r="M7" s="21" t="s">
-        <v>404</v>
-      </c>
-      <c r="N7" s="18" t="s">
-        <v>405</v>
-      </c>
-      <c r="O7" s="18" t="s">
-        <v>406</v>
-      </c>
-      <c r="P7" s="18" t="s">
-        <v>407</v>
-      </c>
-      <c r="Q7" s="18" t="s">
-        <v>408</v>
-      </c>
-      <c r="R7" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="S7" s="22" t="s">
-        <v>410</v>
-      </c>
-      <c r="T7" s="19" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="22" t="s">
+        <v>413</v>
+      </c>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+    </row>
+    <row r="8" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A8" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="19" t="s">
-        <v>412</v>
-      </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="18" t="s">
-        <v>413</v>
-      </c>
-      <c r="M8" s="21" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="21" t="s">
         <v>414</v>
       </c>
-      <c r="N8" s="19" t="s">
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="21" t="s">
         <v>415</v>
       </c>
-      <c r="O8" s="19" t="s">
+      <c r="M8" s="24" t="s">
         <v>416</v>
       </c>
+      <c r="N8" s="21" t="s">
+        <v>417</v>
+      </c>
+      <c r="O8" s="21" t="s">
+        <v>418</v>
+      </c>
       <c r="P8" s="21" t="s">
-        <v>417</v>
-      </c>
-      <c r="Q8" s="18" t="s">
-        <v>418</v>
-      </c>
-      <c r="R8" s="18" t="s">
         <v>419</v>
       </c>
-      <c r="S8" s="18" t="s">
+      <c r="Q8" s="21" t="s">
         <v>420</v>
       </c>
-      <c r="T8" s="18" t="s">
+      <c r="R8" s="21" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="9" spans="1:20" ht="345" x14ac:dyDescent="0.15">
+      <c r="S8" s="25" t="s">
+        <v>422</v>
+      </c>
+      <c r="T8" s="22" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="s">
         <v>325</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="20" t="s">
-        <v>422</v>
-      </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="19" t="s">
-        <v>423</v>
-      </c>
-      <c r="O9" s="17"/>
-      <c r="P9" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="22" t="s">
         <v>424</v>
       </c>
-      <c r="Q9" s="20" t="s">
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="21" t="s">
         <v>425</v>
       </c>
-      <c r="R9" s="20" t="s">
+      <c r="M9" s="24" t="s">
         <v>426</v>
       </c>
-      <c r="S9" s="20" t="s">
+      <c r="N9" s="22" t="s">
         <v>427</v>
       </c>
-      <c r="T9" s="19" t="s">
+      <c r="O9" s="22" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="P9" s="24" t="s">
+        <v>429</v>
+      </c>
+      <c r="Q9" s="21" t="s">
+        <v>430</v>
+      </c>
+      <c r="R9" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="S9" s="21" t="s">
+        <v>432</v>
+      </c>
+      <c r="T9" s="21" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A10" s="4" t="s">
         <v>325</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="18" t="s">
-        <v>429</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>430</v>
-      </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="18" t="s">
-        <v>431</v>
-      </c>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="18" t="s">
-        <v>432</v>
-      </c>
-      <c r="O10" s="17"/>
-      <c r="P10" s="23" t="s">
-        <v>433</v>
-      </c>
-      <c r="Q10" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="23" t="s">
         <v>434</v>
       </c>
-      <c r="R10" s="17"/>
-      <c r="S10" s="17"/>
-      <c r="T10" s="18" t="s">
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="20"/>
+      <c r="M10" s="20"/>
+      <c r="N10" s="22" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" ht="293" x14ac:dyDescent="0.15">
+      <c r="O10" s="20"/>
+      <c r="P10" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="Q10" s="23" t="s">
+        <v>437</v>
+      </c>
+      <c r="R10" s="23" t="s">
+        <v>438</v>
+      </c>
+      <c r="S10" s="23" t="s">
+        <v>439</v>
+      </c>
+      <c r="T10" s="22" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>325</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="20" t="s">
-        <v>437</v>
-      </c>
-      <c r="O11" s="20" t="s">
-        <v>438</v>
-      </c>
-      <c r="P11" s="20" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q11" s="17"/>
-      <c r="R11" s="18" t="s">
-        <v>440</v>
-      </c>
-      <c r="S11" s="17"/>
-      <c r="T11" s="17"/>
-    </row>
-    <row r="12" spans="1:20" ht="154" x14ac:dyDescent="0.15">
+        <v>58</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>442</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="G11" s="21" t="s">
+        <v>443</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="21" t="s">
+        <v>444</v>
+      </c>
+      <c r="O11" s="20"/>
+      <c r="P11" s="26" t="s">
+        <v>445</v>
+      </c>
+      <c r="Q11" s="21" t="s">
+        <v>446</v>
+      </c>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
+      <c r="T11" s="21" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A12" s="4" t="s">
-        <v>336</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="19" t="s">
-        <v>441</v>
-      </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="19" t="s">
-        <v>442</v>
-      </c>
-      <c r="M12" s="21" t="s">
-        <v>443</v>
-      </c>
-      <c r="N12" s="19" t="s">
-        <v>444</v>
-      </c>
-      <c r="O12" s="19" t="s">
-        <v>445</v>
-      </c>
-      <c r="P12" s="21" t="s">
-        <v>446</v>
-      </c>
-      <c r="Q12" s="19" t="s">
-        <v>447</v>
-      </c>
-      <c r="R12" s="19" t="s">
+        <v>325</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="S12" s="19" t="s">
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="23" t="s">
         <v>449</v>
       </c>
-      <c r="T12" s="19" t="s">
+      <c r="O12" s="23" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="13" spans="1:20" ht="210" x14ac:dyDescent="0.15">
+      <c r="P12" s="23" t="s">
+        <v>451</v>
+      </c>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="S12" s="20"/>
+      <c r="T12" s="20"/>
+    </row>
+    <row r="13" spans="1:21" ht="224" x14ac:dyDescent="0.15">
       <c r="A13" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>451</v>
-      </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="19" t="s">
-        <v>452</v>
-      </c>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="19" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="22" t="s">
         <v>453</v>
       </c>
-      <c r="M13" s="21" t="s">
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="22" t="s">
         <v>454</v>
       </c>
-      <c r="N13" s="19" t="s">
+      <c r="M13" s="24" t="s">
         <v>455</v>
       </c>
-      <c r="O13" s="19" t="s">
+      <c r="N13" s="22" t="s">
         <v>456</v>
       </c>
-      <c r="P13" s="21" t="s">
+      <c r="O13" s="22" t="s">
         <v>457</v>
       </c>
-      <c r="Q13" s="19" t="s">
+      <c r="P13" s="24" t="s">
         <v>458</v>
       </c>
-      <c r="R13" s="18" t="s">
+      <c r="Q13" s="22" t="s">
         <v>459</v>
       </c>
-      <c r="S13" s="18" t="s">
+      <c r="R13" s="22" t="s">
         <v>460</v>
       </c>
-      <c r="T13" s="19" t="s">
+      <c r="S13" s="22" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="14" spans="1:20" ht="358" x14ac:dyDescent="0.15">
+      <c r="T13" s="22" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="306" x14ac:dyDescent="0.15">
       <c r="A14" s="4" t="s">
         <v>336</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19" t="s">
-        <v>462</v>
-      </c>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="19" t="s">
         <v>463</v>
       </c>
-      <c r="M14" s="21" t="s">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="22" t="s">
         <v>464</v>
       </c>
-      <c r="N14" s="19" t="s">
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="22" t="s">
         <v>465</v>
       </c>
-      <c r="O14" s="20" t="s">
+      <c r="M14" s="24" t="s">
         <v>466</v>
       </c>
-      <c r="P14" s="21" t="s">
+      <c r="N14" s="22" t="s">
         <v>467</v>
       </c>
-      <c r="Q14" s="19" t="s">
+      <c r="O14" s="22" t="s">
         <v>468</v>
       </c>
-      <c r="R14" s="20" t="s">
+      <c r="P14" s="24" t="s">
         <v>469</v>
       </c>
-      <c r="S14" s="19" t="s">
+      <c r="Q14" s="22" t="s">
         <v>470</v>
       </c>
-      <c r="T14" s="19" t="s">
+      <c r="R14" s="21" t="s">
         <v>471</v>
       </c>
-    </row>
-    <row r="15" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="S14" s="21" t="s">
+        <v>472</v>
+      </c>
+      <c r="T14" s="22" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A15" s="4" t="s">
         <v>336</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="22" t="s">
+        <v>474</v>
+      </c>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="M15" s="24" t="s">
+        <v>476</v>
+      </c>
+      <c r="N15" s="22" t="s">
+        <v>477</v>
+      </c>
+      <c r="O15" s="23" t="s">
+        <v>478</v>
+      </c>
+      <c r="P15" s="24" t="s">
+        <v>479</v>
+      </c>
+      <c r="Q15" s="22" t="s">
+        <v>480</v>
+      </c>
+      <c r="R15" s="23" t="s">
+        <v>481</v>
+      </c>
+      <c r="S15" s="22" t="s">
+        <v>482</v>
+      </c>
+      <c r="T15" s="22" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="A16" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="18" t="s">
-        <v>472</v>
-      </c>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="18" t="s">
-        <v>473</v>
-      </c>
-      <c r="M15" s="21" t="s">
-        <v>474</v>
-      </c>
-      <c r="N15" s="19" t="s">
-        <v>475</v>
-      </c>
-      <c r="O15" s="19" t="s">
-        <v>476</v>
-      </c>
-      <c r="P15" s="21" t="s">
-        <v>477</v>
-      </c>
-      <c r="Q15" s="23" t="s">
-        <v>478</v>
-      </c>
-      <c r="R15" s="18" t="s">
-        <v>479</v>
-      </c>
-      <c r="S15" s="18" t="s">
-        <v>480</v>
-      </c>
-      <c r="T15" s="19" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" ht="358" x14ac:dyDescent="0.15">
-      <c r="A16" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="19" t="s">
-        <v>482</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>483</v>
-      </c>
-      <c r="E16" s="19" t="s">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="21" t="s">
         <v>484</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="21" t="s">
         <v>485</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="M16" s="24" t="s">
         <v>486</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="N16" s="22" t="s">
         <v>487</v>
       </c>
-      <c r="I16" s="19" t="s">
+      <c r="O16" s="22" t="s">
         <v>488</v>
       </c>
-      <c r="J16" s="19" t="s">
+      <c r="P16" s="24" t="s">
         <v>489</v>
       </c>
-      <c r="K16" s="19" t="s">
+      <c r="Q16" s="26" t="s">
         <v>490</v>
       </c>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="17"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="17"/>
-    </row>
-    <row r="17" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="R16" s="21" t="s">
+        <v>491</v>
+      </c>
+      <c r="S16" s="21" t="s">
+        <v>492</v>
+      </c>
+      <c r="T16" s="22" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="358" x14ac:dyDescent="0.15">
       <c r="A17" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>491</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>492</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>493</v>
-      </c>
-      <c r="E17" s="19" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="22" t="s">
         <v>494</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="D17" s="22" t="s">
         <v>495</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="E17" s="22" t="s">
         <v>496</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="F17" s="22" t="s">
         <v>497</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="G17" s="22" t="s">
         <v>498</v>
       </c>
-      <c r="J17" s="19" t="s">
+      <c r="H17" s="22" t="s">
         <v>499</v>
       </c>
-      <c r="K17" s="19" t="s">
+      <c r="I17" s="22" t="s">
         <v>500</v>
       </c>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-    </row>
-    <row r="18" spans="1:20" ht="358" x14ac:dyDescent="0.15">
+      <c r="J17" s="22" t="s">
+        <v>501</v>
+      </c>
+      <c r="K17" s="22" t="s">
+        <v>502</v>
+      </c>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="20"/>
+      <c r="Q17" s="20"/>
+      <c r="R17" s="20"/>
+      <c r="S17" s="20"/>
+      <c r="T17" s="20"/>
+    </row>
+    <row r="18" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A18" s="4" t="s">
         <v>347</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>502</v>
-      </c>
-      <c r="E18" s="19" t="s">
         <v>503</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>504</v>
       </c>
-      <c r="G18" s="21" t="s">
+      <c r="D18" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="H18" s="21" t="s">
+      <c r="E18" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="I18" s="21" t="s">
+      <c r="F18" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="J18" s="21" t="s">
+      <c r="G18" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="K18" s="18" t="s">
+      <c r="H18" s="22" t="s">
         <v>509</v>
       </c>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
-    </row>
-    <row r="19" spans="1:20" ht="371" x14ac:dyDescent="0.15">
+      <c r="I18" s="22" t="s">
+        <v>510</v>
+      </c>
+      <c r="J18" s="22" t="s">
+        <v>511</v>
+      </c>
+      <c r="K18" s="22" t="s">
+        <v>512</v>
+      </c>
+      <c r="L18" s="20"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="20"/>
+      <c r="P18" s="20"/>
+      <c r="Q18" s="20"/>
+      <c r="R18" s="20"/>
+      <c r="S18" s="20"/>
+      <c r="T18" s="20"/>
+    </row>
+    <row r="19" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A19" s="4" t="s">
         <v>347</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>513</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>514</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>515</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>516</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>517</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>518</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>519</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>520</v>
+      </c>
+      <c r="K19" s="21" t="s">
+        <v>521</v>
+      </c>
+      <c r="L19" s="20"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="20"/>
+      <c r="Q19" s="20"/>
+      <c r="R19" s="20"/>
+      <c r="S19" s="20"/>
+      <c r="T19" s="20"/>
+    </row>
+    <row r="20" spans="1:20" ht="371" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>510</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>511</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>512</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>513</v>
-      </c>
-      <c r="G19" s="19" t="s">
-        <v>514</v>
-      </c>
-      <c r="H19" s="18" t="s">
-        <v>515</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>516</v>
-      </c>
-      <c r="J19" s="18" t="s">
-        <v>517</v>
-      </c>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="17"/>
-    </row>
-    <row r="20" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
-      <c r="A20" s="4" t="s">
-        <v>518</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="18" t="s">
-        <v>520</v>
-      </c>
-      <c r="L20" s="19" t="s">
-        <v>521</v>
-      </c>
-      <c r="M20" s="19" t="s">
+      <c r="C20" s="21" t="s">
         <v>522</v>
       </c>
-      <c r="N20" s="19" t="s">
+      <c r="D20" s="21" t="s">
         <v>523</v>
       </c>
-      <c r="O20" s="19" t="s">
+      <c r="E20" s="22" t="s">
         <v>524</v>
       </c>
-      <c r="P20" s="20" t="s">
+      <c r="F20" s="21" t="s">
         <v>525</v>
       </c>
-      <c r="Q20" s="19" t="s">
+      <c r="G20" s="22" t="s">
         <v>526</v>
       </c>
-      <c r="R20" s="20" t="s">
+      <c r="H20" s="21" t="s">
         <v>527</v>
       </c>
-      <c r="S20" s="19" t="s">
+      <c r="I20" s="22" t="s">
         <v>528</v>
       </c>
-      <c r="T20" s="19" t="s">
+      <c r="J20" s="21" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="21" spans="1:20" ht="319" x14ac:dyDescent="0.15">
+      <c r="K20" s="20"/>
+      <c r="L20" s="20"/>
+      <c r="M20" s="20"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="20"/>
+      <c r="P20" s="20"/>
+      <c r="Q20" s="20"/>
+      <c r="R20" s="20"/>
+      <c r="S20" s="20"/>
+      <c r="T20" s="20"/>
+    </row>
+    <row r="21" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A21" s="4" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="19" t="s">
         <v>530</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="27" t="s">
         <v>531</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="F21" s="21" t="s">
         <v>532</v>
       </c>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="18" t="s">
+      <c r="G21" s="21" t="s">
         <v>533</v>
       </c>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="21" t="s">
+        <v>534</v>
+      </c>
+      <c r="K21" s="21" t="s">
+        <v>535</v>
+      </c>
+      <c r="L21" s="22" t="s">
+        <v>536</v>
+      </c>
+      <c r="M21" s="28" t="s">
+        <v>537</v>
+      </c>
+      <c r="N21" s="28" t="s">
+        <v>538</v>
+      </c>
+      <c r="O21" s="28" t="s">
+        <v>539</v>
+      </c>
+      <c r="P21" s="23" t="s">
+        <v>540</v>
+      </c>
+      <c r="Q21" s="28" t="s">
+        <v>541</v>
+      </c>
+      <c r="R21" s="22" t="s">
+        <v>542</v>
+      </c>
+      <c r="S21" s="22" t="s">
+        <v>543</v>
+      </c>
+      <c r="T21" s="28" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="22" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A22" s="4" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>535</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>536</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>537</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>538</v>
-      </c>
-      <c r="F22" s="19" t="s">
-        <v>539</v>
-      </c>
-      <c r="G22" s="19" t="s">
-        <v>540</v>
-      </c>
-      <c r="H22" s="19" t="s">
-        <v>541</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>542</v>
-      </c>
-      <c r="J22" s="18" t="s">
-        <v>543</v>
-      </c>
-      <c r="K22" s="19" t="s">
-        <v>544</v>
-      </c>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="17"/>
-    </row>
-    <row r="23" spans="1:20" ht="371" x14ac:dyDescent="0.15">
+        <v>282</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="22" t="s">
+        <v>545</v>
+      </c>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="21" t="s">
+        <v>546</v>
+      </c>
+      <c r="L22" s="22" t="s">
+        <v>547</v>
+      </c>
+      <c r="M22" s="22" t="s">
+        <v>548</v>
+      </c>
+      <c r="N22" s="22" t="s">
+        <v>549</v>
+      </c>
+      <c r="O22" s="22" t="s">
+        <v>550</v>
+      </c>
+      <c r="P22" s="23" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q22" s="22" t="s">
+        <v>552</v>
+      </c>
+      <c r="R22" s="23" t="s">
+        <v>553</v>
+      </c>
+      <c r="S22" s="22" t="s">
+        <v>554</v>
+      </c>
+      <c r="T22" s="22" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>382</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>545</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>546</v>
-      </c>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18" t="s">
-        <v>547</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>548</v>
-      </c>
-      <c r="H23" s="17"/>
-      <c r="I23" s="19" t="s">
-        <v>549</v>
-      </c>
-      <c r="J23" s="19" t="s">
-        <v>550</v>
-      </c>
-      <c r="K23" s="17"/>
-      <c r="L23" s="19" t="s">
-        <v>551</v>
-      </c>
-      <c r="M23" s="19" t="s">
-        <v>552</v>
-      </c>
-      <c r="N23" s="17"/>
-      <c r="O23" s="19" t="s">
-        <v>553</v>
-      </c>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="18" t="s">
-        <v>554</v>
-      </c>
-      <c r="R23" s="17"/>
-      <c r="S23" s="19" t="s">
-        <v>555</v>
-      </c>
-      <c r="T23" s="17"/>
-    </row>
-    <row r="24" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+        <v>74</v>
+      </c>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>557</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="21" t="s">
+        <v>559</v>
+      </c>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20"/>
+      <c r="P23" s="20"/>
+      <c r="Q23" s="20"/>
+      <c r="R23" s="20"/>
+      <c r="S23" s="20"/>
+      <c r="T23" s="20"/>
+    </row>
+    <row r="24" spans="1:20" ht="306" x14ac:dyDescent="0.15">
       <c r="A24" s="4" t="s">
-        <v>534</v>
+        <v>560</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>556</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>557</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>558</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>559</v>
-      </c>
-      <c r="G24" s="19" t="s">
         <v>560</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="C24" s="22" t="s">
         <v>561</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="D24" s="28" t="s">
         <v>562</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="E24" s="28" t="s">
         <v>563</v>
       </c>
-      <c r="K24" s="19" t="s">
+      <c r="F24" s="29" t="s">
         <v>564</v>
       </c>
-      <c r="L24" s="19" t="s">
+      <c r="G24" s="22" t="s">
         <v>565</v>
       </c>
-      <c r="M24" s="19" t="s">
+      <c r="H24" s="28" t="s">
         <v>566</v>
       </c>
-      <c r="N24" s="19" t="s">
+      <c r="I24" s="22" t="s">
         <v>567</v>
       </c>
-      <c r="O24" s="19" t="s">
+      <c r="J24" s="4"/>
+      <c r="K24" s="28" t="s">
         <v>568</v>
       </c>
-      <c r="P24" s="20" t="s">
+      <c r="L24" s="28" t="s">
         <v>569</v>
       </c>
-      <c r="Q24" s="20" t="s">
+      <c r="M24" s="30" t="s">
         <v>570</v>
       </c>
-      <c r="R24" s="20" t="s">
+      <c r="N24" s="28" t="s">
         <v>571</v>
       </c>
-      <c r="S24" s="19" t="s">
+      <c r="O24" s="28" t="s">
         <v>572</v>
       </c>
-      <c r="T24" s="20" t="s">
+      <c r="P24" s="23" t="s">
         <v>573</v>
+      </c>
+      <c r="Q24" s="28" t="s">
+        <v>574</v>
+      </c>
+      <c r="R24" s="22" t="s">
+        <v>575</v>
+      </c>
+      <c r="S24" s="22" t="s">
+        <v>576</v>
+      </c>
+      <c r="T24" s="28" t="s">
+        <v>577</v>
       </c>
     </row>
     <row r="25" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
-        <v>534</v>
+        <v>560</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>574</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>575</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>576</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>577</v>
-      </c>
-      <c r="F25" s="20" t="s">
         <v>578</v>
       </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="20" t="s">
+      <c r="C25" s="22" t="s">
         <v>579</v>
       </c>
-      <c r="M25" s="19" t="s">
+      <c r="D25" s="21" t="s">
         <v>580</v>
       </c>
-      <c r="N25" s="19" t="s">
+      <c r="E25" s="21" t="s">
         <v>581</v>
       </c>
-      <c r="O25" s="17"/>
-      <c r="P25" s="20" t="s">
+      <c r="F25" s="21" t="s">
         <v>582</v>
       </c>
-      <c r="Q25" s="20" t="s">
+      <c r="G25" s="22" t="s">
         <v>583</v>
       </c>
-      <c r="R25" s="20" t="s">
+      <c r="H25" s="22" t="s">
         <v>584</v>
       </c>
-      <c r="S25" s="20" t="s">
+      <c r="I25" s="22" t="s">
         <v>585</v>
       </c>
-      <c r="T25" s="20" t="s">
+      <c r="J25" s="22" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" ht="50.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="28" spans="1:20" ht="98.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="30" spans="1:20" ht="55.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="31" spans="1:20" ht="13" x14ac:dyDescent="0.15">
-      <c r="F31" s="24"/>
+      <c r="K25" s="22" t="s">
+        <v>587</v>
+      </c>
+      <c r="L25" s="20"/>
+      <c r="M25" s="20"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="20"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="20"/>
+      <c r="S25" s="20"/>
+      <c r="T25" s="20"/>
+    </row>
+    <row r="26" spans="1:20" ht="371" x14ac:dyDescent="0.15">
+      <c r="A26" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>588</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>589</v>
+      </c>
+      <c r="E26" s="20"/>
+      <c r="F26" s="21" t="s">
+        <v>590</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>591</v>
+      </c>
+      <c r="H26" s="20"/>
+      <c r="I26" s="22" t="s">
+        <v>592</v>
+      </c>
+      <c r="J26" s="22" t="s">
+        <v>593</v>
+      </c>
+      <c r="K26" s="20"/>
+      <c r="L26" s="22" t="s">
+        <v>594</v>
+      </c>
+      <c r="M26" s="22" t="s">
+        <v>595</v>
+      </c>
+      <c r="N26" s="20"/>
+      <c r="O26" s="22" t="s">
+        <v>596</v>
+      </c>
+      <c r="P26" s="20"/>
+      <c r="Q26" s="21" t="s">
+        <v>597</v>
+      </c>
+      <c r="R26" s="20"/>
+      <c r="S26" s="22" t="s">
+        <v>598</v>
+      </c>
+      <c r="T26" s="20"/>
+    </row>
+    <row r="27" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="A27" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>599</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>600</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>601</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>602</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>603</v>
+      </c>
+      <c r="H27" s="22" t="s">
+        <v>604</v>
+      </c>
+      <c r="I27" s="22" t="s">
+        <v>605</v>
+      </c>
+      <c r="J27" s="22" t="s">
+        <v>606</v>
+      </c>
+      <c r="K27" s="22" t="s">
+        <v>607</v>
+      </c>
+      <c r="L27" s="22" t="s">
+        <v>608</v>
+      </c>
+      <c r="M27" s="22" t="s">
+        <v>609</v>
+      </c>
+      <c r="N27" s="22" t="s">
+        <v>610</v>
+      </c>
+      <c r="O27" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="P27" s="23" t="s">
+        <v>612</v>
+      </c>
+      <c r="Q27" s="23" t="s">
+        <v>613</v>
+      </c>
+      <c r="R27" s="23" t="s">
+        <v>614</v>
+      </c>
+      <c r="S27" s="22" t="s">
+        <v>615</v>
+      </c>
+      <c r="T27" s="23" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" ht="409.6" x14ac:dyDescent="0.15">
+      <c r="A28" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>618</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>619</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>620</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>621</v>
+      </c>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="23" t="s">
+        <v>622</v>
+      </c>
+      <c r="M28" s="22" t="s">
+        <v>623</v>
+      </c>
+      <c r="N28" s="22" t="s">
+        <v>624</v>
+      </c>
+      <c r="O28" s="20"/>
+      <c r="P28" s="23" t="s">
+        <v>625</v>
+      </c>
+      <c r="Q28" s="23" t="s">
+        <v>626</v>
+      </c>
+      <c r="R28" s="23" t="s">
+        <v>627</v>
+      </c>
+      <c r="S28" s="23" t="s">
+        <v>628</v>
+      </c>
+      <c r="T28" s="23" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" ht="13" x14ac:dyDescent="0.15">
+      <c r="S29" s="31" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" ht="98.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="33" spans="6:6" ht="55.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="34" spans="6:6" ht="13" x14ac:dyDescent="0.15">
+      <c r="F34" s="32"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="T1:U1"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="M3" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="E4" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
-    <hyperlink ref="L4" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
-    <hyperlink ref="M4" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
-    <hyperlink ref="N4" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
-    <hyperlink ref="O4" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
-    <hyperlink ref="P4" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
-    <hyperlink ref="Q4" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
-    <hyperlink ref="R4" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
-    <hyperlink ref="S4" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
-    <hyperlink ref="T4" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
-    <hyperlink ref="M5" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
-    <hyperlink ref="N5" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
-    <hyperlink ref="P5" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
-    <hyperlink ref="Q6" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
-    <hyperlink ref="E7" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
-    <hyperlink ref="L7" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
-    <hyperlink ref="M7" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
-    <hyperlink ref="N7" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
-    <hyperlink ref="O7" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
-    <hyperlink ref="P7" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
-    <hyperlink ref="Q7" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
-    <hyperlink ref="R7" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
-    <hyperlink ref="S7" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
-    <hyperlink ref="T7" r:id="rId25" xr:uid="{00000000-0004-0000-0200-000018000000}"/>
-    <hyperlink ref="E8" r:id="rId26" xr:uid="{00000000-0004-0000-0200-000019000000}"/>
-    <hyperlink ref="L8" r:id="rId27" xr:uid="{00000000-0004-0000-0200-00001A000000}"/>
-    <hyperlink ref="M8" r:id="rId28" xr:uid="{00000000-0004-0000-0200-00001B000000}"/>
-    <hyperlink ref="N8" r:id="rId29" xr:uid="{00000000-0004-0000-0200-00001C000000}"/>
-    <hyperlink ref="O8" r:id="rId30" xr:uid="{00000000-0004-0000-0200-00001D000000}"/>
-    <hyperlink ref="P8" r:id="rId31" xr:uid="{00000000-0004-0000-0200-00001E000000}"/>
-    <hyperlink ref="Q8" r:id="rId32" xr:uid="{00000000-0004-0000-0200-00001F000000}"/>
-    <hyperlink ref="R8" r:id="rId33" xr:uid="{00000000-0004-0000-0200-000020000000}"/>
-    <hyperlink ref="S8" r:id="rId34" xr:uid="{00000000-0004-0000-0200-000021000000}"/>
-    <hyperlink ref="T8" r:id="rId35" xr:uid="{00000000-0004-0000-0200-000022000000}"/>
-    <hyperlink ref="G9" r:id="rId36" xr:uid="{00000000-0004-0000-0200-000023000000}"/>
-    <hyperlink ref="N9" r:id="rId37" xr:uid="{00000000-0004-0000-0200-000024000000}"/>
-    <hyperlink ref="P9" r:id="rId38" xr:uid="{00000000-0004-0000-0200-000025000000}"/>
-    <hyperlink ref="Q9" r:id="rId39" xr:uid="{00000000-0004-0000-0200-000026000000}"/>
-    <hyperlink ref="R9" r:id="rId40" xr:uid="{00000000-0004-0000-0200-000027000000}"/>
-    <hyperlink ref="S9" r:id="rId41" xr:uid="{00000000-0004-0000-0200-000028000000}"/>
-    <hyperlink ref="T9" r:id="rId42" xr:uid="{00000000-0004-0000-0200-000029000000}"/>
-    <hyperlink ref="D10" r:id="rId43" xr:uid="{00000000-0004-0000-0200-00002A000000}"/>
-    <hyperlink ref="E10" r:id="rId44" xr:uid="{00000000-0004-0000-0200-00002B000000}"/>
-    <hyperlink ref="G10" r:id="rId45" xr:uid="{00000000-0004-0000-0200-00002C000000}"/>
-    <hyperlink ref="N10" r:id="rId46" xr:uid="{00000000-0004-0000-0200-00002D000000}"/>
-    <hyperlink ref="Q10" r:id="rId47" xr:uid="{00000000-0004-0000-0200-00002E000000}"/>
-    <hyperlink ref="T10" r:id="rId48" xr:uid="{00000000-0004-0000-0200-00002F000000}"/>
-    <hyperlink ref="N11" r:id="rId49" xr:uid="{00000000-0004-0000-0200-000030000000}"/>
-    <hyperlink ref="O11" r:id="rId50" xr:uid="{00000000-0004-0000-0200-000031000000}"/>
-    <hyperlink ref="P11" r:id="rId51" xr:uid="{00000000-0004-0000-0200-000032000000}"/>
-    <hyperlink ref="R11" r:id="rId52" xr:uid="{00000000-0004-0000-0200-000033000000}"/>
-    <hyperlink ref="E12" r:id="rId53" xr:uid="{00000000-0004-0000-0200-000034000000}"/>
-    <hyperlink ref="L12" r:id="rId54" xr:uid="{00000000-0004-0000-0200-000035000000}"/>
-    <hyperlink ref="M12" r:id="rId55" xr:uid="{00000000-0004-0000-0200-000036000000}"/>
-    <hyperlink ref="N12" r:id="rId56" xr:uid="{00000000-0004-0000-0200-000037000000}"/>
-    <hyperlink ref="O12" r:id="rId57" xr:uid="{00000000-0004-0000-0200-000038000000}"/>
-    <hyperlink ref="P12" r:id="rId58" xr:uid="{00000000-0004-0000-0200-000039000000}"/>
-    <hyperlink ref="Q12" r:id="rId59" xr:uid="{00000000-0004-0000-0200-00003A000000}"/>
-    <hyperlink ref="R12" r:id="rId60" xr:uid="{00000000-0004-0000-0200-00003B000000}"/>
-    <hyperlink ref="S12" r:id="rId61" xr:uid="{00000000-0004-0000-0200-00003C000000}"/>
-    <hyperlink ref="T12" r:id="rId62" xr:uid="{00000000-0004-0000-0200-00003D000000}"/>
-    <hyperlink ref="E13" r:id="rId63" xr:uid="{00000000-0004-0000-0200-00003E000000}"/>
-    <hyperlink ref="L13" r:id="rId64" xr:uid="{00000000-0004-0000-0200-00003F000000}"/>
-    <hyperlink ref="M13" r:id="rId65" xr:uid="{00000000-0004-0000-0200-000040000000}"/>
-    <hyperlink ref="N13" r:id="rId66" xr:uid="{00000000-0004-0000-0200-000041000000}"/>
-    <hyperlink ref="O13" r:id="rId67" xr:uid="{00000000-0004-0000-0200-000042000000}"/>
-    <hyperlink ref="P13" r:id="rId68" xr:uid="{00000000-0004-0000-0200-000043000000}"/>
-    <hyperlink ref="Q13" r:id="rId69" xr:uid="{00000000-0004-0000-0200-000044000000}"/>
-    <hyperlink ref="R13" r:id="rId70" xr:uid="{00000000-0004-0000-0200-000045000000}"/>
-    <hyperlink ref="S13" r:id="rId71" xr:uid="{00000000-0004-0000-0200-000046000000}"/>
-    <hyperlink ref="T13" r:id="rId72" xr:uid="{00000000-0004-0000-0200-000047000000}"/>
-    <hyperlink ref="E14" r:id="rId73" xr:uid="{00000000-0004-0000-0200-000048000000}"/>
-    <hyperlink ref="L14" r:id="rId74" xr:uid="{00000000-0004-0000-0200-000049000000}"/>
-    <hyperlink ref="M14" r:id="rId75" xr:uid="{00000000-0004-0000-0200-00004A000000}"/>
-    <hyperlink ref="N14" r:id="rId76" xr:uid="{00000000-0004-0000-0200-00004B000000}"/>
-    <hyperlink ref="O14" r:id="rId77" xr:uid="{00000000-0004-0000-0200-00004C000000}"/>
-    <hyperlink ref="P14" r:id="rId78" xr:uid="{00000000-0004-0000-0200-00004D000000}"/>
-    <hyperlink ref="Q14" r:id="rId79" xr:uid="{00000000-0004-0000-0200-00004E000000}"/>
-    <hyperlink ref="R14" r:id="rId80" xr:uid="{00000000-0004-0000-0200-00004F000000}"/>
-    <hyperlink ref="S14" r:id="rId81" xr:uid="{00000000-0004-0000-0200-000050000000}"/>
-    <hyperlink ref="T14" r:id="rId82" xr:uid="{00000000-0004-0000-0200-000051000000}"/>
-    <hyperlink ref="E15" r:id="rId83" xr:uid="{00000000-0004-0000-0200-000052000000}"/>
-    <hyperlink ref="L15" r:id="rId84" xr:uid="{00000000-0004-0000-0200-000053000000}"/>
-    <hyperlink ref="M15" r:id="rId85" xr:uid="{00000000-0004-0000-0200-000054000000}"/>
-    <hyperlink ref="N15" r:id="rId86" xr:uid="{00000000-0004-0000-0200-000055000000}"/>
-    <hyperlink ref="O15" r:id="rId87" xr:uid="{00000000-0004-0000-0200-000056000000}"/>
-    <hyperlink ref="P15" r:id="rId88" xr:uid="{00000000-0004-0000-0200-000057000000}"/>
-    <hyperlink ref="R15" r:id="rId89" xr:uid="{00000000-0004-0000-0200-000058000000}"/>
-    <hyperlink ref="S15" r:id="rId90" xr:uid="{00000000-0004-0000-0200-000059000000}"/>
-    <hyperlink ref="T15" r:id="rId91" xr:uid="{00000000-0004-0000-0200-00005A000000}"/>
-    <hyperlink ref="C16" r:id="rId92" xr:uid="{00000000-0004-0000-0200-00005B000000}"/>
-    <hyperlink ref="D16" r:id="rId93" xr:uid="{00000000-0004-0000-0200-00005C000000}"/>
-    <hyperlink ref="E16" r:id="rId94" xr:uid="{00000000-0004-0000-0200-00005D000000}"/>
-    <hyperlink ref="F16" r:id="rId95" xr:uid="{00000000-0004-0000-0200-00005E000000}"/>
-    <hyperlink ref="G16" r:id="rId96" xr:uid="{00000000-0004-0000-0200-00005F000000}"/>
-    <hyperlink ref="H16" r:id="rId97" xr:uid="{00000000-0004-0000-0200-000060000000}"/>
-    <hyperlink ref="I16" r:id="rId98" xr:uid="{00000000-0004-0000-0200-000061000000}"/>
-    <hyperlink ref="J16" r:id="rId99" xr:uid="{00000000-0004-0000-0200-000062000000}"/>
-    <hyperlink ref="K16" r:id="rId100" xr:uid="{00000000-0004-0000-0200-000063000000}"/>
-    <hyperlink ref="C17" r:id="rId101" xr:uid="{00000000-0004-0000-0200-000064000000}"/>
-    <hyperlink ref="D17" r:id="rId102" xr:uid="{00000000-0004-0000-0200-000065000000}"/>
-    <hyperlink ref="E17" r:id="rId103" xr:uid="{00000000-0004-0000-0200-000066000000}"/>
-    <hyperlink ref="F17" r:id="rId104" xr:uid="{00000000-0004-0000-0200-000067000000}"/>
-    <hyperlink ref="G17" r:id="rId105" xr:uid="{00000000-0004-0000-0200-000068000000}"/>
-    <hyperlink ref="H17" r:id="rId106" xr:uid="{00000000-0004-0000-0200-000069000000}"/>
-    <hyperlink ref="I17" r:id="rId107" xr:uid="{00000000-0004-0000-0200-00006A000000}"/>
-    <hyperlink ref="J17" r:id="rId108" xr:uid="{00000000-0004-0000-0200-00006B000000}"/>
-    <hyperlink ref="K17" r:id="rId109" xr:uid="{00000000-0004-0000-0200-00006C000000}"/>
-    <hyperlink ref="C18" r:id="rId110" xr:uid="{00000000-0004-0000-0200-00006D000000}"/>
-    <hyperlink ref="D18" r:id="rId111" xr:uid="{00000000-0004-0000-0200-00006E000000}"/>
-    <hyperlink ref="E18" r:id="rId112" xr:uid="{00000000-0004-0000-0200-00006F000000}"/>
-    <hyperlink ref="F18" r:id="rId113" xr:uid="{00000000-0004-0000-0200-000070000000}"/>
-    <hyperlink ref="G18" r:id="rId114" xr:uid="{00000000-0004-0000-0200-000071000000}"/>
-    <hyperlink ref="H18" r:id="rId115" xr:uid="{00000000-0004-0000-0200-000072000000}"/>
-    <hyperlink ref="I18" r:id="rId116" xr:uid="{00000000-0004-0000-0200-000073000000}"/>
-    <hyperlink ref="J18" r:id="rId117" xr:uid="{00000000-0004-0000-0200-000074000000}"/>
-    <hyperlink ref="K18" r:id="rId118" xr:uid="{00000000-0004-0000-0200-000075000000}"/>
-    <hyperlink ref="C19" r:id="rId119" xr:uid="{00000000-0004-0000-0200-000076000000}"/>
-    <hyperlink ref="D19" r:id="rId120" xr:uid="{00000000-0004-0000-0200-000077000000}"/>
-    <hyperlink ref="E19" r:id="rId121" xr:uid="{00000000-0004-0000-0200-000078000000}"/>
-    <hyperlink ref="F19" r:id="rId122" xr:uid="{00000000-0004-0000-0200-000079000000}"/>
-    <hyperlink ref="G19" r:id="rId123" xr:uid="{00000000-0004-0000-0200-00007A000000}"/>
-    <hyperlink ref="H19" r:id="rId124" xr:uid="{00000000-0004-0000-0200-00007B000000}"/>
-    <hyperlink ref="I19" r:id="rId125" xr:uid="{00000000-0004-0000-0200-00007C000000}"/>
-    <hyperlink ref="J19" r:id="rId126" xr:uid="{00000000-0004-0000-0200-00007D000000}"/>
-    <hyperlink ref="E20" r:id="rId127" xr:uid="{00000000-0004-0000-0200-00007E000000}"/>
-    <hyperlink ref="K20" r:id="rId128" xr:uid="{00000000-0004-0000-0200-00007F000000}"/>
-    <hyperlink ref="L20" r:id="rId129" xr:uid="{00000000-0004-0000-0200-000080000000}"/>
-    <hyperlink ref="M20" r:id="rId130" xr:uid="{00000000-0004-0000-0200-000081000000}"/>
-    <hyperlink ref="N20" r:id="rId131" xr:uid="{00000000-0004-0000-0200-000082000000}"/>
-    <hyperlink ref="O20" r:id="rId132" xr:uid="{00000000-0004-0000-0200-000083000000}"/>
-    <hyperlink ref="P20" r:id="rId133" xr:uid="{00000000-0004-0000-0200-000084000000}"/>
-    <hyperlink ref="Q20" r:id="rId134" xr:uid="{00000000-0004-0000-0200-000085000000}"/>
-    <hyperlink ref="R20" r:id="rId135" xr:uid="{00000000-0004-0000-0200-000086000000}"/>
-    <hyperlink ref="S20" r:id="rId136" xr:uid="{00000000-0004-0000-0200-000087000000}"/>
-    <hyperlink ref="T20" r:id="rId137" xr:uid="{00000000-0004-0000-0200-000088000000}"/>
-    <hyperlink ref="E21" r:id="rId138" xr:uid="{00000000-0004-0000-0200-000089000000}"/>
-    <hyperlink ref="F21" r:id="rId139" xr:uid="{00000000-0004-0000-0200-00008A000000}"/>
-    <hyperlink ref="G21" r:id="rId140" xr:uid="{00000000-0004-0000-0200-00008B000000}"/>
-    <hyperlink ref="J21" r:id="rId141" xr:uid="{00000000-0004-0000-0200-00008C000000}"/>
-    <hyperlink ref="C22" r:id="rId142" xr:uid="{00000000-0004-0000-0200-00008D000000}"/>
-    <hyperlink ref="D22" r:id="rId143" xr:uid="{00000000-0004-0000-0200-00008E000000}"/>
-    <hyperlink ref="E22" r:id="rId144" xr:uid="{00000000-0004-0000-0200-00008F000000}"/>
-    <hyperlink ref="F22" r:id="rId145" xr:uid="{00000000-0004-0000-0200-000090000000}"/>
-    <hyperlink ref="G22" r:id="rId146" xr:uid="{00000000-0004-0000-0200-000091000000}"/>
-    <hyperlink ref="H22" r:id="rId147" xr:uid="{00000000-0004-0000-0200-000092000000}"/>
-    <hyperlink ref="I22" r:id="rId148" xr:uid="{00000000-0004-0000-0200-000093000000}"/>
-    <hyperlink ref="J22" r:id="rId149" xr:uid="{00000000-0004-0000-0200-000094000000}"/>
-    <hyperlink ref="K22" r:id="rId150" xr:uid="{00000000-0004-0000-0200-000095000000}"/>
-    <hyperlink ref="C23" r:id="rId151" xr:uid="{00000000-0004-0000-0200-000096000000}"/>
-    <hyperlink ref="D23" r:id="rId152" xr:uid="{00000000-0004-0000-0200-000097000000}"/>
-    <hyperlink ref="F23" r:id="rId153" xr:uid="{00000000-0004-0000-0200-000098000000}"/>
-    <hyperlink ref="G23" r:id="rId154" xr:uid="{00000000-0004-0000-0200-000099000000}"/>
-    <hyperlink ref="I23" r:id="rId155" xr:uid="{00000000-0004-0000-0200-00009A000000}"/>
-    <hyperlink ref="J23" r:id="rId156" xr:uid="{00000000-0004-0000-0200-00009B000000}"/>
-    <hyperlink ref="L23" r:id="rId157" xr:uid="{00000000-0004-0000-0200-00009C000000}"/>
-    <hyperlink ref="M23" r:id="rId158" xr:uid="{00000000-0004-0000-0200-00009D000000}"/>
-    <hyperlink ref="O23" r:id="rId159" xr:uid="{00000000-0004-0000-0200-00009E000000}"/>
-    <hyperlink ref="Q23" r:id="rId160" xr:uid="{00000000-0004-0000-0200-00009F000000}"/>
-    <hyperlink ref="S23" r:id="rId161" xr:uid="{00000000-0004-0000-0200-0000A0000000}"/>
-    <hyperlink ref="C24" r:id="rId162" xr:uid="{00000000-0004-0000-0200-0000A1000000}"/>
-    <hyperlink ref="D24" r:id="rId163" xr:uid="{00000000-0004-0000-0200-0000A2000000}"/>
-    <hyperlink ref="E24" r:id="rId164" xr:uid="{00000000-0004-0000-0200-0000A3000000}"/>
-    <hyperlink ref="F24" r:id="rId165" xr:uid="{00000000-0004-0000-0200-0000A4000000}"/>
-    <hyperlink ref="G24" r:id="rId166" xr:uid="{00000000-0004-0000-0200-0000A5000000}"/>
-    <hyperlink ref="H24" r:id="rId167" xr:uid="{00000000-0004-0000-0200-0000A6000000}"/>
-    <hyperlink ref="I24" r:id="rId168" xr:uid="{00000000-0004-0000-0200-0000A7000000}"/>
-    <hyperlink ref="J24" r:id="rId169" xr:uid="{00000000-0004-0000-0200-0000A8000000}"/>
-    <hyperlink ref="K24" r:id="rId170" xr:uid="{00000000-0004-0000-0200-0000A9000000}"/>
-    <hyperlink ref="L24" r:id="rId171" xr:uid="{00000000-0004-0000-0200-0000AA000000}"/>
-    <hyperlink ref="M24" r:id="rId172" xr:uid="{00000000-0004-0000-0200-0000AB000000}"/>
-    <hyperlink ref="N24" r:id="rId173" xr:uid="{00000000-0004-0000-0200-0000AC000000}"/>
-    <hyperlink ref="O24" r:id="rId174" xr:uid="{00000000-0004-0000-0200-0000AD000000}"/>
-    <hyperlink ref="P24" r:id="rId175" xr:uid="{00000000-0004-0000-0200-0000AE000000}"/>
-    <hyperlink ref="Q24" r:id="rId176" xr:uid="{00000000-0004-0000-0200-0000AF000000}"/>
-    <hyperlink ref="R24" r:id="rId177" xr:uid="{00000000-0004-0000-0200-0000B0000000}"/>
-    <hyperlink ref="S24" r:id="rId178" xr:uid="{00000000-0004-0000-0200-0000B1000000}"/>
-    <hyperlink ref="T24" r:id="rId179" xr:uid="{00000000-0004-0000-0200-0000B2000000}"/>
-    <hyperlink ref="C25" r:id="rId180" xr:uid="{00000000-0004-0000-0200-0000B3000000}"/>
-    <hyperlink ref="D25" r:id="rId181" xr:uid="{00000000-0004-0000-0200-0000B4000000}"/>
-    <hyperlink ref="E25" r:id="rId182" xr:uid="{00000000-0004-0000-0200-0000B5000000}"/>
-    <hyperlink ref="F25" r:id="rId183" xr:uid="{00000000-0004-0000-0200-0000B6000000}"/>
-    <hyperlink ref="L25" r:id="rId184" xr:uid="{00000000-0004-0000-0200-0000B7000000}"/>
-    <hyperlink ref="M25" r:id="rId185" xr:uid="{00000000-0004-0000-0200-0000B8000000}"/>
-    <hyperlink ref="N25" r:id="rId186" xr:uid="{00000000-0004-0000-0200-0000B9000000}"/>
-    <hyperlink ref="P25" r:id="rId187" xr:uid="{00000000-0004-0000-0200-0000BA000000}"/>
-    <hyperlink ref="Q25" r:id="rId188" xr:uid="{00000000-0004-0000-0200-0000BB000000}"/>
-    <hyperlink ref="R25" r:id="rId189" xr:uid="{00000000-0004-0000-0200-0000BC000000}"/>
-    <hyperlink ref="S25" r:id="rId190" xr:uid="{00000000-0004-0000-0200-0000BD000000}"/>
-    <hyperlink ref="T25" r:id="rId191" xr:uid="{00000000-0004-0000-0200-0000BE000000}"/>
+    <hyperlink ref="M4" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="L5" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="M5" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="N5" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="O5" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="P5" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="Q5" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="R5" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="S5" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="T5" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="M6" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="N6" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="P6" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="Q7" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="E8" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
+    <hyperlink ref="L8" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
+    <hyperlink ref="M8" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
+    <hyperlink ref="N8" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
+    <hyperlink ref="O8" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
+    <hyperlink ref="P8" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
+    <hyperlink ref="Q8" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
+    <hyperlink ref="R8" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
+    <hyperlink ref="S8" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
+    <hyperlink ref="T8" r:id="rId25" xr:uid="{00000000-0004-0000-0200-000018000000}"/>
+    <hyperlink ref="E9" r:id="rId26" xr:uid="{00000000-0004-0000-0200-000019000000}"/>
+    <hyperlink ref="L9" r:id="rId27" xr:uid="{00000000-0004-0000-0200-00001A000000}"/>
+    <hyperlink ref="M9" r:id="rId28" xr:uid="{00000000-0004-0000-0200-00001B000000}"/>
+    <hyperlink ref="N9" r:id="rId29" xr:uid="{00000000-0004-0000-0200-00001C000000}"/>
+    <hyperlink ref="O9" r:id="rId30" xr:uid="{00000000-0004-0000-0200-00001D000000}"/>
+    <hyperlink ref="P9" r:id="rId31" xr:uid="{00000000-0004-0000-0200-00001E000000}"/>
+    <hyperlink ref="Q9" r:id="rId32" xr:uid="{00000000-0004-0000-0200-00001F000000}"/>
+    <hyperlink ref="R9" r:id="rId33" xr:uid="{00000000-0004-0000-0200-000020000000}"/>
+    <hyperlink ref="S9" r:id="rId34" xr:uid="{00000000-0004-0000-0200-000021000000}"/>
+    <hyperlink ref="T9" r:id="rId35" xr:uid="{00000000-0004-0000-0200-000022000000}"/>
+    <hyperlink ref="G10" r:id="rId36" xr:uid="{00000000-0004-0000-0200-000023000000}"/>
+    <hyperlink ref="N10" r:id="rId37" xr:uid="{00000000-0004-0000-0200-000024000000}"/>
+    <hyperlink ref="P10" r:id="rId38" xr:uid="{00000000-0004-0000-0200-000025000000}"/>
+    <hyperlink ref="Q10" r:id="rId39" xr:uid="{00000000-0004-0000-0200-000026000000}"/>
+    <hyperlink ref="R10" r:id="rId40" xr:uid="{00000000-0004-0000-0200-000027000000}"/>
+    <hyperlink ref="S10" r:id="rId41" xr:uid="{00000000-0004-0000-0200-000028000000}"/>
+    <hyperlink ref="T10" r:id="rId42" xr:uid="{00000000-0004-0000-0200-000029000000}"/>
+    <hyperlink ref="D11" r:id="rId43" xr:uid="{00000000-0004-0000-0200-00002A000000}"/>
+    <hyperlink ref="E11" r:id="rId44" xr:uid="{00000000-0004-0000-0200-00002B000000}"/>
+    <hyperlink ref="G11" r:id="rId45" xr:uid="{00000000-0004-0000-0200-00002C000000}"/>
+    <hyperlink ref="N11" r:id="rId46" xr:uid="{00000000-0004-0000-0200-00002D000000}"/>
+    <hyperlink ref="Q11" r:id="rId47" xr:uid="{00000000-0004-0000-0200-00002E000000}"/>
+    <hyperlink ref="T11" r:id="rId48" xr:uid="{00000000-0004-0000-0200-00002F000000}"/>
+    <hyperlink ref="N12" r:id="rId49" xr:uid="{00000000-0004-0000-0200-000030000000}"/>
+    <hyperlink ref="O12" r:id="rId50" xr:uid="{00000000-0004-0000-0200-000031000000}"/>
+    <hyperlink ref="P12" r:id="rId51" xr:uid="{00000000-0004-0000-0200-000032000000}"/>
+    <hyperlink ref="R12" r:id="rId52" xr:uid="{00000000-0004-0000-0200-000033000000}"/>
+    <hyperlink ref="E13" r:id="rId53" xr:uid="{00000000-0004-0000-0200-000034000000}"/>
+    <hyperlink ref="L13" r:id="rId54" xr:uid="{00000000-0004-0000-0200-000035000000}"/>
+    <hyperlink ref="M13" r:id="rId55" xr:uid="{00000000-0004-0000-0200-000036000000}"/>
+    <hyperlink ref="N13" r:id="rId56" xr:uid="{00000000-0004-0000-0200-000037000000}"/>
+    <hyperlink ref="O13" r:id="rId57" xr:uid="{00000000-0004-0000-0200-000038000000}"/>
+    <hyperlink ref="P13" r:id="rId58" xr:uid="{00000000-0004-0000-0200-000039000000}"/>
+    <hyperlink ref="Q13" r:id="rId59" xr:uid="{00000000-0004-0000-0200-00003A000000}"/>
+    <hyperlink ref="R13" r:id="rId60" xr:uid="{00000000-0004-0000-0200-00003B000000}"/>
+    <hyperlink ref="S13" r:id="rId61" xr:uid="{00000000-0004-0000-0200-00003C000000}"/>
+    <hyperlink ref="T13" r:id="rId62" xr:uid="{00000000-0004-0000-0200-00003D000000}"/>
+    <hyperlink ref="E14" r:id="rId63" xr:uid="{00000000-0004-0000-0200-00003E000000}"/>
+    <hyperlink ref="L14" r:id="rId64" xr:uid="{00000000-0004-0000-0200-00003F000000}"/>
+    <hyperlink ref="M14" r:id="rId65" xr:uid="{00000000-0004-0000-0200-000040000000}"/>
+    <hyperlink ref="N14" r:id="rId66" xr:uid="{00000000-0004-0000-0200-000041000000}"/>
+    <hyperlink ref="O14" r:id="rId67" xr:uid="{00000000-0004-0000-0200-000042000000}"/>
+    <hyperlink ref="P14" r:id="rId68" xr:uid="{00000000-0004-0000-0200-000043000000}"/>
+    <hyperlink ref="Q14" r:id="rId69" xr:uid="{00000000-0004-0000-0200-000044000000}"/>
+    <hyperlink ref="R14" r:id="rId70" xr:uid="{00000000-0004-0000-0200-000045000000}"/>
+    <hyperlink ref="S14" r:id="rId71" xr:uid="{00000000-0004-0000-0200-000046000000}"/>
+    <hyperlink ref="T14" r:id="rId72" xr:uid="{00000000-0004-0000-0200-000047000000}"/>
+    <hyperlink ref="E15" r:id="rId73" xr:uid="{00000000-0004-0000-0200-000048000000}"/>
+    <hyperlink ref="L15" r:id="rId74" xr:uid="{00000000-0004-0000-0200-000049000000}"/>
+    <hyperlink ref="M15" r:id="rId75" xr:uid="{00000000-0004-0000-0200-00004A000000}"/>
+    <hyperlink ref="N15" r:id="rId76" xr:uid="{00000000-0004-0000-0200-00004B000000}"/>
+    <hyperlink ref="O15" r:id="rId77" xr:uid="{00000000-0004-0000-0200-00004C000000}"/>
+    <hyperlink ref="P15" r:id="rId78" xr:uid="{00000000-0004-0000-0200-00004D000000}"/>
+    <hyperlink ref="Q15" r:id="rId79" xr:uid="{00000000-0004-0000-0200-00004E000000}"/>
+    <hyperlink ref="R15" r:id="rId80" xr:uid="{00000000-0004-0000-0200-00004F000000}"/>
+    <hyperlink ref="S15" r:id="rId81" xr:uid="{00000000-0004-0000-0200-000050000000}"/>
+    <hyperlink ref="T15" r:id="rId82" xr:uid="{00000000-0004-0000-0200-000051000000}"/>
+    <hyperlink ref="E16" r:id="rId83" xr:uid="{00000000-0004-0000-0200-000052000000}"/>
+    <hyperlink ref="L16" r:id="rId84" xr:uid="{00000000-0004-0000-0200-000053000000}"/>
+    <hyperlink ref="M16" r:id="rId85" xr:uid="{00000000-0004-0000-0200-000054000000}"/>
+    <hyperlink ref="N16" r:id="rId86" xr:uid="{00000000-0004-0000-0200-000055000000}"/>
+    <hyperlink ref="O16" r:id="rId87" xr:uid="{00000000-0004-0000-0200-000056000000}"/>
+    <hyperlink ref="P16" r:id="rId88" xr:uid="{00000000-0004-0000-0200-000057000000}"/>
+    <hyperlink ref="R16" r:id="rId89" xr:uid="{00000000-0004-0000-0200-000058000000}"/>
+    <hyperlink ref="S16" r:id="rId90" xr:uid="{00000000-0004-0000-0200-000059000000}"/>
+    <hyperlink ref="T16" r:id="rId91" xr:uid="{00000000-0004-0000-0200-00005A000000}"/>
+    <hyperlink ref="C17" r:id="rId92" xr:uid="{00000000-0004-0000-0200-00005B000000}"/>
+    <hyperlink ref="D17" r:id="rId93" xr:uid="{00000000-0004-0000-0200-00005C000000}"/>
+    <hyperlink ref="E17" r:id="rId94" xr:uid="{00000000-0004-0000-0200-00005D000000}"/>
+    <hyperlink ref="F17" r:id="rId95" xr:uid="{00000000-0004-0000-0200-00005E000000}"/>
+    <hyperlink ref="G17" r:id="rId96" xr:uid="{00000000-0004-0000-0200-00005F000000}"/>
+    <hyperlink ref="H17" r:id="rId97" xr:uid="{00000000-0004-0000-0200-000060000000}"/>
+    <hyperlink ref="I17" r:id="rId98" xr:uid="{00000000-0004-0000-0200-000061000000}"/>
+    <hyperlink ref="J17" r:id="rId99" xr:uid="{00000000-0004-0000-0200-000062000000}"/>
+    <hyperlink ref="K17" r:id="rId100" xr:uid="{00000000-0004-0000-0200-000063000000}"/>
+    <hyperlink ref="C18" r:id="rId101" xr:uid="{00000000-0004-0000-0200-000064000000}"/>
+    <hyperlink ref="D18" r:id="rId102" xr:uid="{00000000-0004-0000-0200-000065000000}"/>
+    <hyperlink ref="E18" r:id="rId103" xr:uid="{00000000-0004-0000-0200-000066000000}"/>
+    <hyperlink ref="F18" r:id="rId104" xr:uid="{00000000-0004-0000-0200-000067000000}"/>
+    <hyperlink ref="G18" r:id="rId105" xr:uid="{00000000-0004-0000-0200-000068000000}"/>
+    <hyperlink ref="H18" r:id="rId106" xr:uid="{00000000-0004-0000-0200-000069000000}"/>
+    <hyperlink ref="I18" r:id="rId107" xr:uid="{00000000-0004-0000-0200-00006A000000}"/>
+    <hyperlink ref="J18" r:id="rId108" xr:uid="{00000000-0004-0000-0200-00006B000000}"/>
+    <hyperlink ref="K18" r:id="rId109" xr:uid="{00000000-0004-0000-0200-00006C000000}"/>
+    <hyperlink ref="C19" r:id="rId110" xr:uid="{00000000-0004-0000-0200-00006D000000}"/>
+    <hyperlink ref="D19" r:id="rId111" xr:uid="{00000000-0004-0000-0200-00006E000000}"/>
+    <hyperlink ref="E19" r:id="rId112" xr:uid="{00000000-0004-0000-0200-00006F000000}"/>
+    <hyperlink ref="F19" r:id="rId113" xr:uid="{00000000-0004-0000-0200-000070000000}"/>
+    <hyperlink ref="G19" r:id="rId114" xr:uid="{00000000-0004-0000-0200-000071000000}"/>
+    <hyperlink ref="H19" r:id="rId115" xr:uid="{00000000-0004-0000-0200-000072000000}"/>
+    <hyperlink ref="I19" r:id="rId116" xr:uid="{00000000-0004-0000-0200-000073000000}"/>
+    <hyperlink ref="J19" r:id="rId117" xr:uid="{00000000-0004-0000-0200-000074000000}"/>
+    <hyperlink ref="K19" r:id="rId118" xr:uid="{00000000-0004-0000-0200-000075000000}"/>
+    <hyperlink ref="C20" r:id="rId119" xr:uid="{00000000-0004-0000-0200-000076000000}"/>
+    <hyperlink ref="D20" r:id="rId120" xr:uid="{00000000-0004-0000-0200-000077000000}"/>
+    <hyperlink ref="E20" r:id="rId121" xr:uid="{00000000-0004-0000-0200-000078000000}"/>
+    <hyperlink ref="F20" r:id="rId122" xr:uid="{00000000-0004-0000-0200-000079000000}"/>
+    <hyperlink ref="G20" r:id="rId123" xr:uid="{00000000-0004-0000-0200-00007A000000}"/>
+    <hyperlink ref="H20" r:id="rId124" xr:uid="{00000000-0004-0000-0200-00007B000000}"/>
+    <hyperlink ref="I20" r:id="rId125" xr:uid="{00000000-0004-0000-0200-00007C000000}"/>
+    <hyperlink ref="J20" r:id="rId126" xr:uid="{00000000-0004-0000-0200-00007D000000}"/>
+    <hyperlink ref="E21" r:id="rId127" xr:uid="{00000000-0004-0000-0200-00007E000000}"/>
+    <hyperlink ref="F21" r:id="rId128" xr:uid="{00000000-0004-0000-0200-00007F000000}"/>
+    <hyperlink ref="G21" r:id="rId129" xr:uid="{00000000-0004-0000-0200-000080000000}"/>
+    <hyperlink ref="J21" r:id="rId130" xr:uid="{00000000-0004-0000-0200-000081000000}"/>
+    <hyperlink ref="K21" r:id="rId131" xr:uid="{00000000-0004-0000-0200-000082000000}"/>
+    <hyperlink ref="L21" r:id="rId132" xr:uid="{00000000-0004-0000-0200-000083000000}"/>
+    <hyperlink ref="P21" r:id="rId133" xr:uid="{00000000-0004-0000-0200-000084000000}"/>
+    <hyperlink ref="R21" r:id="rId134" xr:uid="{00000000-0004-0000-0200-000085000000}"/>
+    <hyperlink ref="S21" r:id="rId135" xr:uid="{00000000-0004-0000-0200-000086000000}"/>
+    <hyperlink ref="E22" r:id="rId136" xr:uid="{00000000-0004-0000-0200-000087000000}"/>
+    <hyperlink ref="K22" r:id="rId137" xr:uid="{00000000-0004-0000-0200-000088000000}"/>
+    <hyperlink ref="L22" r:id="rId138" xr:uid="{00000000-0004-0000-0200-000089000000}"/>
+    <hyperlink ref="M22" r:id="rId139" xr:uid="{00000000-0004-0000-0200-00008A000000}"/>
+    <hyperlink ref="N22" r:id="rId140" xr:uid="{00000000-0004-0000-0200-00008B000000}"/>
+    <hyperlink ref="O22" r:id="rId141" xr:uid="{00000000-0004-0000-0200-00008C000000}"/>
+    <hyperlink ref="P22" r:id="rId142" xr:uid="{00000000-0004-0000-0200-00008D000000}"/>
+    <hyperlink ref="Q22" r:id="rId143" xr:uid="{00000000-0004-0000-0200-00008E000000}"/>
+    <hyperlink ref="R22" r:id="rId144" xr:uid="{00000000-0004-0000-0200-00008F000000}"/>
+    <hyperlink ref="S22" r:id="rId145" xr:uid="{00000000-0004-0000-0200-000090000000}"/>
+    <hyperlink ref="T22" r:id="rId146" xr:uid="{00000000-0004-0000-0200-000091000000}"/>
+    <hyperlink ref="E23" r:id="rId147" xr:uid="{00000000-0004-0000-0200-000092000000}"/>
+    <hyperlink ref="F23" r:id="rId148" xr:uid="{00000000-0004-0000-0200-000093000000}"/>
+    <hyperlink ref="G23" r:id="rId149" xr:uid="{00000000-0004-0000-0200-000094000000}"/>
+    <hyperlink ref="J23" r:id="rId150" xr:uid="{00000000-0004-0000-0200-000095000000}"/>
+    <hyperlink ref="C24" r:id="rId151" xr:uid="{00000000-0004-0000-0200-000096000000}"/>
+    <hyperlink ref="G24" r:id="rId152" xr:uid="{00000000-0004-0000-0200-000097000000}"/>
+    <hyperlink ref="I24" r:id="rId153" xr:uid="{00000000-0004-0000-0200-000098000000}"/>
+    <hyperlink ref="M24" r:id="rId154" xr:uid="{00000000-0004-0000-0200-000099000000}"/>
+    <hyperlink ref="P24" r:id="rId155" xr:uid="{00000000-0004-0000-0200-00009A000000}"/>
+    <hyperlink ref="R24" r:id="rId156" xr:uid="{00000000-0004-0000-0200-00009B000000}"/>
+    <hyperlink ref="S24" r:id="rId157" xr:uid="{00000000-0004-0000-0200-00009C000000}"/>
+    <hyperlink ref="C25" r:id="rId158" xr:uid="{00000000-0004-0000-0200-00009D000000}"/>
+    <hyperlink ref="D25" r:id="rId159" xr:uid="{00000000-0004-0000-0200-00009E000000}"/>
+    <hyperlink ref="E25" r:id="rId160" xr:uid="{00000000-0004-0000-0200-00009F000000}"/>
+    <hyperlink ref="F25" r:id="rId161" xr:uid="{00000000-0004-0000-0200-0000A0000000}"/>
+    <hyperlink ref="G25" r:id="rId162" xr:uid="{00000000-0004-0000-0200-0000A1000000}"/>
+    <hyperlink ref="H25" r:id="rId163" xr:uid="{00000000-0004-0000-0200-0000A2000000}"/>
+    <hyperlink ref="I25" r:id="rId164" xr:uid="{00000000-0004-0000-0200-0000A3000000}"/>
+    <hyperlink ref="J25" r:id="rId165" xr:uid="{00000000-0004-0000-0200-0000A4000000}"/>
+    <hyperlink ref="K25" r:id="rId166" xr:uid="{00000000-0004-0000-0200-0000A5000000}"/>
+    <hyperlink ref="C26" r:id="rId167" xr:uid="{00000000-0004-0000-0200-0000A6000000}"/>
+    <hyperlink ref="D26" r:id="rId168" xr:uid="{00000000-0004-0000-0200-0000A7000000}"/>
+    <hyperlink ref="F26" r:id="rId169" xr:uid="{00000000-0004-0000-0200-0000A8000000}"/>
+    <hyperlink ref="G26" r:id="rId170" xr:uid="{00000000-0004-0000-0200-0000A9000000}"/>
+    <hyperlink ref="I26" r:id="rId171" xr:uid="{00000000-0004-0000-0200-0000AA000000}"/>
+    <hyperlink ref="J26" r:id="rId172" xr:uid="{00000000-0004-0000-0200-0000AB000000}"/>
+    <hyperlink ref="L26" r:id="rId173" xr:uid="{00000000-0004-0000-0200-0000AC000000}"/>
+    <hyperlink ref="M26" r:id="rId174" xr:uid="{00000000-0004-0000-0200-0000AD000000}"/>
+    <hyperlink ref="O26" r:id="rId175" xr:uid="{00000000-0004-0000-0200-0000AE000000}"/>
+    <hyperlink ref="Q26" r:id="rId176" xr:uid="{00000000-0004-0000-0200-0000AF000000}"/>
+    <hyperlink ref="S26" r:id="rId177" xr:uid="{00000000-0004-0000-0200-0000B0000000}"/>
+    <hyperlink ref="C27" r:id="rId178" xr:uid="{00000000-0004-0000-0200-0000B1000000}"/>
+    <hyperlink ref="D27" r:id="rId179" xr:uid="{00000000-0004-0000-0200-0000B2000000}"/>
+    <hyperlink ref="E27" r:id="rId180" xr:uid="{00000000-0004-0000-0200-0000B3000000}"/>
+    <hyperlink ref="F27" r:id="rId181" xr:uid="{00000000-0004-0000-0200-0000B4000000}"/>
+    <hyperlink ref="G27" r:id="rId182" xr:uid="{00000000-0004-0000-0200-0000B5000000}"/>
+    <hyperlink ref="H27" r:id="rId183" xr:uid="{00000000-0004-0000-0200-0000B6000000}"/>
+    <hyperlink ref="I27" r:id="rId184" xr:uid="{00000000-0004-0000-0200-0000B7000000}"/>
+    <hyperlink ref="J27" r:id="rId185" xr:uid="{00000000-0004-0000-0200-0000B8000000}"/>
+    <hyperlink ref="K27" r:id="rId186" xr:uid="{00000000-0004-0000-0200-0000B9000000}"/>
+    <hyperlink ref="L27" r:id="rId187" xr:uid="{00000000-0004-0000-0200-0000BA000000}"/>
+    <hyperlink ref="M27" r:id="rId188" xr:uid="{00000000-0004-0000-0200-0000BB000000}"/>
+    <hyperlink ref="N27" r:id="rId189" xr:uid="{00000000-0004-0000-0200-0000BC000000}"/>
+    <hyperlink ref="O27" r:id="rId190" xr:uid="{00000000-0004-0000-0200-0000BD000000}"/>
+    <hyperlink ref="P27" r:id="rId191" xr:uid="{00000000-0004-0000-0200-0000BE000000}"/>
+    <hyperlink ref="Q27" r:id="rId192" xr:uid="{00000000-0004-0000-0200-0000BF000000}"/>
+    <hyperlink ref="R27" r:id="rId193" xr:uid="{00000000-0004-0000-0200-0000C0000000}"/>
+    <hyperlink ref="S27" r:id="rId194" xr:uid="{00000000-0004-0000-0200-0000C1000000}"/>
+    <hyperlink ref="T27" r:id="rId195" xr:uid="{00000000-0004-0000-0200-0000C2000000}"/>
+    <hyperlink ref="C28" r:id="rId196" xr:uid="{00000000-0004-0000-0200-0000C3000000}"/>
+    <hyperlink ref="D28" r:id="rId197" xr:uid="{00000000-0004-0000-0200-0000C4000000}"/>
+    <hyperlink ref="E28" r:id="rId198" xr:uid="{00000000-0004-0000-0200-0000C5000000}"/>
+    <hyperlink ref="F28" r:id="rId199" xr:uid="{00000000-0004-0000-0200-0000C6000000}"/>
+    <hyperlink ref="L28" r:id="rId200" xr:uid="{00000000-0004-0000-0200-0000C7000000}"/>
+    <hyperlink ref="M28" r:id="rId201" xr:uid="{00000000-0004-0000-0200-0000C8000000}"/>
+    <hyperlink ref="N28" r:id="rId202" xr:uid="{00000000-0004-0000-0200-0000C9000000}"/>
+    <hyperlink ref="P28" r:id="rId203" xr:uid="{00000000-0004-0000-0200-0000CA000000}"/>
+    <hyperlink ref="Q28" r:id="rId204" xr:uid="{00000000-0004-0000-0200-0000CB000000}"/>
+    <hyperlink ref="R28" r:id="rId205" xr:uid="{00000000-0004-0000-0200-0000CC000000}"/>
+    <hyperlink ref="S28" r:id="rId206" xr:uid="{00000000-0004-0000-0200-0000CD000000}"/>
+    <hyperlink ref="T28" r:id="rId207" xr:uid="{00000000-0004-0000-0200-0000CE000000}"/>
+    <hyperlink ref="S29" r:id="rId208" xr:uid="{00000000-0004-0000-0200-0000CF000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>